<commit_message>
recipes: resolve risky intake policy
</commit_message>
<xml_diff>
--- a/tmp/recipe_intake/cleaned_recipes.xlsx
+++ b/tmp/recipe_intake/cleaned_recipes.xlsx
@@ -2394,7 +2394,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Реалистичное фото: салат с помидорами «Красное море» на простой тарелке, видны помидоры, крабовые палочки, твердый сыр, яйцо, зелень, естественный дневной свет, без текста, логотипов и людей.</t>
+          <t>Реалистичное фото: салат с помидорами «Красное море» на простой тарелке, видны помидоры, крабовые палочки, твердый сыр, яйцо, греческий йогурт, зелень, естественный дневной свет, без текста, логотипов и людей.</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
@@ -3636,7 +3636,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Стручковая фасоль с чесноком и соевым соусом: основное блюдо на 1 порцию с стручковая фасоль, яйцо или тофу, рис сухой, чеснок.</t>
+          <t>Стручковая фасоль с чесноком и соевым соусом: основное блюдо на 1 порцию с стручковая фасоль, тофу, рис сухой, чеснок.</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -3670,12 +3670,12 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>main, simple, растительный белок</t>
+          <t>main, simple, без яиц, растительный белок</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>Реалистичное фото: стручковая фасоль с чесноком и соевым соусом на простой тарелке, видны стручковая фасоль, рис сухой, яйцо или тофу, чеснок, соевый соус, естественный дневной свет, без текста, логотипов и людей.</t>
+          <t>Реалистичное фото: стручковая фасоль с чесноком и соевым соусом на простой тарелке, видны стручковая фасоль, рис сухой, тофу, чеснок, соевый соус, естественный дневной свет, без текста, логотипов и людей.</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr">
@@ -5527,7 +5527,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Курица с овощами по-деревенски: основное блюдо на 1 порцию с филе бедра курицы, смесь овощная «Три капусты», тыква кубиками «Айс», масло оливковое.</t>
+          <t>Курица с овощами по-деревенски: основное блюдо на 1 порцию с филе бедра курицы, смесь овощная «Три капусты», мускатная тыква кубиками, масло оливковое.</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>Реалистичное фото: курица с овощами по-деревенски на простой тарелке, видны филе бедра курицы, смесь овощная «Три капусты», тыква кубиками «Айс», масло оливковое, сливки 20%, естественный дневной свет, без текста, логотипов и людей.</t>
+          <t>Реалистичное фото: курица с овощами по-деревенски на простой тарелке, видны филе бедра курицы, смесь овощная «Три капусты», мускатная тыква кубиками, масло оливковое, сливки 20%, естественный дневной свет, без текста, логотипов и людей.</t>
         </is>
       </c>
       <c r="M85" s="2" t="inlineStr">
@@ -5832,12 +5832,12 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Рулет из лаваша с хумусом: основное блюдо на 1 порцию с хумус, лаваш, вяленые томаты, салат айсберг.</t>
+          <t>Рулет из лаваша с хумусом: перекус / light meal на 1 порцию с хумус, лаваш, вяленые томаты, салат айсберг.</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>snack</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -5866,7 +5866,7 @@
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t>main, simple, без яиц, без молочки, без готовки</t>
+          <t>snack, simple, без яиц, без молочки, без готовки, растительный белок</t>
         </is>
       </c>
       <c r="L90" s="2" t="inlineStr">
@@ -6198,7 +6198,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Салат с шампиньонами и спаржей: перекус на 1 порцию с стручковая фасоль, пекинская капуста, шампиньоны, виноград кишмиш.</t>
+          <t>Салат с шампиньонами и спаржей: перекус на 1 порцию с спаржа, пекинская капуста, шампиньоны, виноград кишмиш.</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -6232,12 +6232,12 @@
       </c>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t>snack, simple, без яиц, без молочки, растительный белок</t>
+          <t>snack, simple, без яиц, без молочки</t>
         </is>
       </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>Реалистичное фото: салат с шампиньонами и спаржей на простой тарелке, видны пекинская капуста, шампиньоны, стручковая фасоль, виноград кишмиш, грецкие орехи, естественный дневной свет, без текста, логотипов и людей.</t>
+          <t>Реалистичное фото: салат с шампиньонами и спаржей на простой тарелке, видны пекинская капуста, шампиньоны, спаржа, виноград кишмиш, грецкие орехи, естественный дневной свет, без текста, логотипов и людей.</t>
         </is>
       </c>
       <c r="M96" s="2" t="inlineStr">
@@ -6381,7 +6381,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Паста с консервированным тунцом и томатами: основное блюдо на 1 порцию с тунец консервированный, сливочный сыр, паста, томаты черри.</t>
+          <t>Паста с консервированным тунцом и томатами: основное блюдо на 1 порцию с тунец консервированный, сливочный сыр, паста, помидоры черри.</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="L99" s="2" t="inlineStr">
         <is>
-          <t>Реалистичное фото: паста с консервированным тунцом и томатами на простой тарелке, видны паста, томаты черри, протертые томаты, тунец консервированный, оливковое масло, естественный дневной свет, без текста, логотипов и людей.</t>
+          <t>Реалистичное фото: паста с консервированным тунцом и томатами на простой тарелке, видны паста, помидоры черри, пассата, тунец консервированный, оливковое масло, естественный дневной свет, без текста, логотипов и людей.</t>
         </is>
       </c>
       <c r="M99" s="2" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Паста болоньезе: основное блюдо на 1 порцию с говяжий фарш, макароны, томатный соус, чеснок.</t>
+          <t>Паста болоньезе: основное блюдо на 1 порцию с говяжий фарш, макароны, пассата, чеснок.</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -6542,7 +6542,7 @@
       </c>
       <c r="L101" s="2" t="inlineStr">
         <is>
-          <t>Реалистичное фото: паста болоньезе на простой тарелке, видны макароны, говяжий фарш, томатный соус, чеснок, лук, естественный дневной свет, без текста, логотипов и людей.</t>
+          <t>Реалистичное фото: паста болоньезе на простой тарелке, видны макароны, говяжий фарш, пассата, чеснок, лук, естественный дневной свет, без текста, логотипов и людей.</t>
         </is>
       </c>
       <c r="M101" s="2" t="inlineStr">
@@ -6559,12 +6559,12 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Паста с куриными колбасками в остром томатном соусе</t>
+          <t>Паста с куриным филе в остром томатном соусе</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Паста с куриными колбасками в остром томатном соусе: основное блюдо на 1 порцию с куриные колбаски, макароны, томатный соус аррабиата, оливковое масло.</t>
+          <t>Паста с куриным филе в остром томатном соусе: основное блюдо на 1 порцию с куриное филе, макароны, пассата, оливковое масло.</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -6603,7 +6603,7 @@
       </c>
       <c r="L102" s="2" t="inlineStr">
         <is>
-          <t>Реалистичное фото: паста с куриными колбасками в остром томатном соусе на простой тарелке, видны макароны, куриные колбаски, томатный соус аррабиата, оливковое масло, сладкий перец, естественный дневной свет, без текста, логотипов и людей.</t>
+          <t>Реалистичное фото: паста с куриным филе в остром томатном соусе на простой тарелке, видны макароны, куриное филе, пассата, оливковое масло, сладкий перец, естественный дневной свет, без текста, логотипов и людей.</t>
         </is>
       </c>
       <c r="M102" s="2" t="inlineStr">
@@ -10881,7 +10881,7 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>reconstructed from title; cod liver mapping confirmed by user decision</t>
+          <t>reconstructed from title; cod liver mapping confirmed by user decision; cod liver canned/drained mapping readiness confirmed; no extra jar oil unless recipe explicitly uses oil; not a future scalable protein anchor</t>
         </is>
       </c>
     </row>
@@ -11839,7 +11839,7 @@
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>amount inferred</t>
+          <t>amount inferred; standard soy sauce condiment policy approved by user; sodium can remain low-confidence note</t>
         </is>
       </c>
     </row>
@@ -12093,7 +12093,7 @@
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
-          <t>amount inferred; dry buckwheat mapping confirmed by user decision</t>
+          <t>amount inferred; dry buckwheat mapping confirmed by user decision; dry buckwheat mapping readiness confirmed by user decision</t>
         </is>
       </c>
     </row>
@@ -12801,7 +12801,7 @@
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>cod liver mapping confirmed by user decision</t>
+          <t>cod liver mapping confirmed by user decision; cod liver canned/drained mapping readiness confirmed; no extra jar oil unless recipe explicitly uses oil; not a future scalable protein anchor</t>
         </is>
       </c>
     </row>
@@ -12995,7 +12995,7 @@
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
-          <t>cod liver mapping confirmed by user decision</t>
+          <t>cod liver mapping confirmed by user decision; cod liver canned/drained mapping readiness confirmed; no extra jar oil unless recipe explicitly uses oil; not a future scalable protein anchor</t>
         </is>
       </c>
     </row>
@@ -13189,7 +13189,7 @@
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
-          <t>cod liver mapping confirmed by user decision</t>
+          <t>cod liver mapping confirmed by user decision; cod liver canned/drained mapping readiness confirmed; no extra jar oil unless recipe explicitly uses oil; not a future scalable protein anchor</t>
         </is>
       </c>
     </row>
@@ -13319,7 +13319,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H186" s="2" t="n"/>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>generic mayo policy approved by user because grams are explicit; high-fat/low-confidence note acceptable</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
@@ -13385,7 +13389,7 @@
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
-          <t>cod liver mapping confirmed by user decision</t>
+          <t>cod liver mapping confirmed by user decision; cod liver canned/drained mapping readiness confirmed; no extra jar oil unless recipe explicitly uses oil; not a future scalable protein anchor</t>
         </is>
       </c>
     </row>
@@ -13545,7 +13549,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H193" s="2" t="n"/>
+      <c r="H193" s="2" t="inlineStr">
+        <is>
+          <t>generic mayo policy approved by user because grams are explicit; high-fat/low-confidence note acceptable</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -13613,7 +13621,7 @@
       </c>
       <c r="H195" s="2" t="inlineStr">
         <is>
-          <t>cod liver mapping confirmed by user decision</t>
+          <t>cod liver mapping confirmed by user decision; cod liver canned/drained mapping readiness confirmed; no extra jar oil unless recipe explicitly uses oil; not a future scalable protein anchor</t>
         </is>
       </c>
     </row>
@@ -13809,7 +13817,7 @@
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
-          <t>normalized in validated cleanup slice</t>
+          <t>normalized in validated cleanup slice; generic mayo policy approved by user because grams are explicit; high-fat/low-confidence note acceptable</t>
         </is>
       </c>
     </row>
@@ -13877,7 +13885,7 @@
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
-          <t>fresh grape mapping confirmed by user decision</t>
+          <t>fresh grape mapping confirmed by user decision; fresh grape/kishmish mapping readiness confirmed; avoid beverage-alias substring matching</t>
         </is>
       </c>
     </row>
@@ -14615,7 +14623,7 @@
       </c>
       <c r="H226" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>scaled from source; generic crab sticks mapping/product policy approved by user</t>
         </is>
       </c>
     </row>
@@ -14779,7 +14787,7 @@
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>майонез или йогурт</t>
+          <t>греческий йогурт</t>
         </is>
       </c>
       <c r="C231" s="2" t="n">
@@ -14805,7 +14813,7 @@
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>dressing normalized to yogurt by user decision; generic yogurt mapping readiness confirmed</t>
         </is>
       </c>
     </row>
@@ -15267,7 +15275,7 @@
       </c>
       <c r="H244" s="2" t="inlineStr">
         <is>
-          <t>cornmeal/polenta mapping confirmed by user decision</t>
+          <t>cornmeal/polenta mapping confirmed by user decision; cornmeal/polenta mapping readiness confirmed by user decision</t>
         </is>
       </c>
     </row>
@@ -17781,7 +17789,7 @@
       </c>
       <c r="H319" s="2" t="inlineStr">
         <is>
-          <t>turkey liver replaced with chicken liver by user decision</t>
+          <t>turkey liver replaced with chicken liver by user decision; chicken liver mapping readiness confirmed by user decision</t>
         </is>
       </c>
     </row>
@@ -18107,7 +18115,7 @@
       </c>
       <c r="H328" s="2" t="inlineStr">
         <is>
-          <t>scaled from source; dry buckwheat mapping confirmed by user decision</t>
+          <t>scaled from source; dry buckwheat mapping confirmed by user decision; dry buckwheat mapping readiness confirmed by user decision</t>
         </is>
       </c>
     </row>
@@ -19369,15 +19377,15 @@
       </c>
       <c r="B367" s="2" t="inlineStr">
         <is>
-          <t>яйцо или тофу</t>
+          <t>тофу</t>
         </is>
       </c>
       <c r="C367" s="2" t="n">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E367" s="2" t="n">
@@ -19385,7 +19393,7 @@
       </c>
       <c r="F367" s="2" t="inlineStr">
         <is>
-          <t>по желанию для белка</t>
+          <t>кубиками</t>
         </is>
       </c>
       <c r="G367" s="2" t="inlineStr">
@@ -19395,7 +19403,7 @@
       </c>
       <c r="H367" s="2" t="inlineStr">
         <is>
-          <t>added to make main meal usable</t>
+          <t>egg/tofu ambiguity resolved to tofu by user decision; tofu-only protein anchor</t>
         </is>
       </c>
     </row>
@@ -19467,7 +19475,7 @@
       </c>
       <c r="H369" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>scaled from source; standard soy sauce condiment policy approved by user; sodium can remain low-confidence note</t>
         </is>
       </c>
     </row>
@@ -19607,7 +19615,7 @@
       </c>
       <c r="H373" s="2" t="inlineStr">
         <is>
-          <t>scaled from source; chicken liver mapping confirmed by user decision</t>
+          <t>scaled from source; chicken liver mapping confirmed by user decision; chicken liver mapping readiness confirmed by user decision</t>
         </is>
       </c>
     </row>
@@ -22323,7 +22331,7 @@
       </c>
       <c r="B459" s="2" t="inlineStr">
         <is>
-          <t>хмели-сунели</t>
+          <t>специи</t>
         </is>
       </c>
       <c r="C459" s="2" t="inlineStr">
@@ -22339,13 +22347,21 @@
       <c r="E459" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F459" s="2" t="n"/>
+      <c r="F459" s="2" t="inlineStr">
+        <is>
+          <t>хмели-сунели</t>
+        </is>
+      </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H459" s="2" t="n"/>
+      <c r="H459" s="2" t="inlineStr">
+        <is>
+          <t>khmeli-suneli mapped to mixed_spices by user decision</t>
+        </is>
+      </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
@@ -22853,7 +22869,7 @@
       </c>
       <c r="H475" s="2" t="inlineStr">
         <is>
-          <t>normalized in validated cleanup slice</t>
+          <t>normalized in validated cleanup slice; standard soy sauce condiment policy approved by user; sodium can remain low-confidence note</t>
         </is>
       </c>
     </row>
@@ -24975,7 +24991,7 @@
       </c>
       <c r="H540" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>scaled from source; standard soy sauce condiment policy approved by user; sodium can remain low-confidence note</t>
         </is>
       </c>
     </row>
@@ -25085,7 +25101,7 @@
       </c>
       <c r="H543" s="2" t="inlineStr">
         <is>
-          <t>split pea mapping confirmed by user decision</t>
+          <t>split pea mapping confirmed by user decision; split peas mapping readiness confirmed by user decision</t>
         </is>
       </c>
     </row>
@@ -25373,7 +25389,7 @@
       </c>
       <c r="H552" s="2" t="inlineStr">
         <is>
-          <t>normalized in validated cleanup slice</t>
+          <t>normalized in validated cleanup slice; teriyaki policy approved with modest explicit grams; low-confidence sodium/sugar note acceptable</t>
         </is>
       </c>
     </row>
@@ -26853,7 +26869,7 @@
       </c>
       <c r="H596" s="2" t="inlineStr">
         <is>
-          <t>trout mapping confirmed by user decision</t>
+          <t>trout mapping confirmed by user decision; trout mapping readiness confirmed by user decision</t>
         </is>
       </c>
     </row>
@@ -27009,7 +27025,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H601" s="2" t="n"/>
+      <c r="H601" s="2" t="inlineStr">
+        <is>
+          <t>pesto policy approved with explicit grams; low-confidence prepared sauce note acceptable</t>
+        </is>
+      </c>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
@@ -27696,7 +27716,7 @@
       </c>
       <c r="B624" s="2" t="inlineStr">
         <is>
-          <t>лапша удон для быстрого приготовления</t>
+          <t>лапша удон</t>
         </is>
       </c>
       <c r="C624" s="2" t="n">
@@ -27710,7 +27730,11 @@
       <c r="E624" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="F624" s="2" t="n"/>
+      <c r="F624" s="2" t="inlineStr">
+        <is>
+          <t>generic udon noodles</t>
+        </is>
+      </c>
       <c r="G624" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -27718,7 +27742,7 @@
       </c>
       <c r="H624" s="2" t="inlineStr">
         <is>
-          <t>from source; normalized in validated cleanup slice</t>
+          <t>product-specific udon wording removed by user decision; generic udon mapping readiness marked</t>
         </is>
       </c>
     </row>
@@ -27976,7 +28000,7 @@
       </c>
       <c r="H631" s="2" t="inlineStr">
         <is>
-          <t>from source</t>
+          <t>from source; standard soy sauce condiment policy approved by user; sodium can remain low-confidence note</t>
         </is>
       </c>
     </row>
@@ -28096,7 +28120,7 @@
       </c>
       <c r="B635" s="2" t="inlineStr">
         <is>
-          <t>рис басмати</t>
+          <t>рис</t>
         </is>
       </c>
       <c r="C635" s="2" t="n">
@@ -28110,13 +28134,21 @@
       <c r="E635" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="F635" s="2" t="n"/>
+      <c r="F635" s="2" t="inlineStr">
+        <is>
+          <t>басмати</t>
+        </is>
+      </c>
       <c r="G635" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H635" s="2" t="n"/>
+      <c r="H635" s="2" t="inlineStr">
+        <is>
+          <t>basmati rice mapping readiness confirmed by user decision; mapped through rice/basmati policy</t>
+        </is>
+      </c>
     </row>
     <row r="636">
       <c r="A636" s="2" t="inlineStr">
@@ -28922,7 +28954,7 @@
       </c>
       <c r="B661" s="2" t="inlineStr">
         <is>
-          <t>тыква кубиками «Айс»</t>
+          <t>мускатная тыква</t>
         </is>
       </c>
       <c r="C661" s="2" t="n">
@@ -28936,13 +28968,21 @@
       <c r="E661" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="F661" s="2" t="n"/>
+      <c r="F661" s="2" t="inlineStr">
+        <is>
+          <t>кубиками, generic raw pumpkin; brand removed</t>
+        </is>
+      </c>
       <c r="G661" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H661" s="2" t="n"/>
+      <c r="H661" s="2" t="inlineStr">
+        <is>
+          <t>branded/frozen pumpkin normalized to generic pumpkin cubes by user decision</t>
+        </is>
+      </c>
     </row>
     <row r="662">
       <c r="A662" s="2" t="inlineStr">
@@ -29190,7 +29230,7 @@
       </c>
       <c r="H669" s="2" t="inlineStr">
         <is>
-          <t>normalized in validated cleanup slice</t>
+          <t>normalized in validated cleanup slice; standard soy sauce condiment policy approved by user; sodium can remain low-confidence note</t>
         </is>
       </c>
     </row>
@@ -29296,7 +29336,7 @@
       </c>
       <c r="H672" s="2" t="inlineStr">
         <is>
-          <t>normalized in validated cleanup slice</t>
+          <t>normalized in validated cleanup slice; canned/chopped tomatoes mapping readiness confirmed by user-approved tomato variant policy</t>
         </is>
       </c>
     </row>
@@ -29536,7 +29576,7 @@
       </c>
       <c r="B680" s="2" t="inlineStr">
         <is>
-          <t>свиные отбивные</t>
+          <t>свиная отбивная</t>
         </is>
       </c>
       <c r="C680" s="2" t="n">
@@ -29558,7 +29598,7 @@
       </c>
       <c r="H680" s="2" t="inlineStr">
         <is>
-          <t>normalized in validated cleanup slice</t>
+          <t>plural pork chops mapped to pork_chop by user decision</t>
         </is>
       </c>
     </row>
@@ -29738,7 +29778,7 @@
       </c>
       <c r="B686" s="2" t="inlineStr">
         <is>
-          <t>приправа для овощей или универсальная</t>
+          <t>специи</t>
         </is>
       </c>
       <c r="C686" s="2" t="inlineStr">
@@ -29751,14 +29791,24 @@
           <t>по вкусу</t>
         </is>
       </c>
-      <c r="E686" s="2" t="n"/>
-      <c r="F686" s="2" t="n"/>
+      <c r="E686" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F686" s="2" t="inlineStr">
+        <is>
+          <t>для овощей/универсальная; 0g seasoning policy</t>
+        </is>
+      </c>
       <c r="G686" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H686" s="2" t="n"/>
+      <c r="H686" s="2" t="inlineStr">
+        <is>
+          <t>universal seasoning mapped to mixed_spices/0g seasoning by user decision</t>
+        </is>
+      </c>
     </row>
     <row r="687">
       <c r="A687" s="2" t="inlineStr">
@@ -30347,12 +30397,12 @@
       <c r="F704" s="2" t="n"/>
       <c r="G704" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H704" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>scaled from source; hummus accepted as weak/low-confidence plant protein anchor for snack/light meal</t>
         </is>
       </c>
     </row>
@@ -30386,7 +30436,7 @@
       </c>
       <c r="H705" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>scaled from source; sun-dried tomato mapping readiness confirmed by user decision</t>
         </is>
       </c>
     </row>
@@ -31428,7 +31478,7 @@
       </c>
       <c r="H737" s="2" t="inlineStr">
         <is>
-          <t>frozen/prepared falafel mapping readiness confirmed by user decision; plant protein anchor</t>
+          <t>frozen/prepared falafel mapping readiness confirmed by user decision; plant protein anchor; frozen/prepared falafel mapping policy approved as generic prepared product; plant protein anchor low-confidence</t>
         </is>
       </c>
     </row>
@@ -31528,7 +31578,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H740" s="2" t="n"/>
+      <c r="H740" s="2" t="inlineStr">
+        <is>
+          <t>prepared Korean carrot remains low-confidence unless accepted as generic carrot/prepared vegetable</t>
+        </is>
+      </c>
     </row>
     <row r="741">
       <c r="A741" s="2" t="inlineStr">
@@ -31658,7 +31712,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H744" s="2" t="n"/>
+      <c r="H744" s="2" t="inlineStr">
+        <is>
+          <t>large prepared mayo-soy sauce remains high-fat/low-confidence; future preview may decompose to generic mayo + soy sauce</t>
+        </is>
+      </c>
     </row>
     <row r="745">
       <c r="A745" s="2" t="inlineStr">
@@ -31820,7 +31878,7 @@
       </c>
       <c r="H749" s="2" t="inlineStr">
         <is>
-          <t>blue cheese replaced with gouda by user decision</t>
+          <t>strong cheese variant replaced with gouda by user decision</t>
         </is>
       </c>
     </row>
@@ -31938,7 +31996,7 @@
       </c>
       <c r="B753" s="2" t="inlineStr">
         <is>
-          <t>стручковая фасоль</t>
+          <t>спаржа</t>
         </is>
       </c>
       <c r="C753" s="2" t="n">
@@ -31954,17 +32012,17 @@
       </c>
       <c r="F753" s="2" t="inlineStr">
         <is>
-          <t>вместо спаржи</t>
+          <t>восстановлено вместо green beans</t>
         </is>
       </c>
       <c r="G753" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H753" s="2" t="inlineStr">
         <is>
-          <t>accessible replacement</t>
+          <t>asparagus restored by user decision; asparagus mapping readiness confirmed</t>
         </is>
       </c>
     </row>
@@ -31998,7 +32056,7 @@
       </c>
       <c r="H754" s="2" t="inlineStr">
         <is>
-          <t>from source; fresh kishmish grape mapping confirmed by user decision</t>
+          <t>from source; fresh kishmish grape mapping confirmed by user decision; fresh grape/kishmish mapping readiness confirmed; avoid beverage-alias substring matching</t>
         </is>
       </c>
     </row>
@@ -32332,7 +32390,7 @@
       </c>
       <c r="B764" s="2" t="inlineStr">
         <is>
-          <t>яичные желтки</t>
+          <t>яичный желток</t>
         </is>
       </c>
       <c r="C764" s="2" t="n">
@@ -32354,7 +32412,7 @@
       </c>
       <c r="H764" s="2" t="inlineStr">
         <is>
-          <t>from source; normalized in validated cleanup slice</t>
+          <t>plural egg yolks mapped to egg_yolk by user decision</t>
         </is>
       </c>
     </row>
@@ -32664,7 +32722,7 @@
       </c>
       <c r="B774" s="2" t="inlineStr">
         <is>
-          <t>томаты черри</t>
+          <t>помидоры черри</t>
         </is>
       </c>
       <c r="C774" s="2" t="n">
@@ -32680,7 +32738,7 @@
       </c>
       <c r="F774" s="2" t="inlineStr">
         <is>
-          <t>половинками</t>
+          <t>половинками; maps to tomato policy</t>
         </is>
       </c>
       <c r="G774" s="2" t="inlineStr">
@@ -32690,7 +32748,7 @@
       </c>
       <c r="H774" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>cherry tomatoes mapped to tomato by user-approved tomato variant policy</t>
         </is>
       </c>
     </row>
@@ -32702,7 +32760,7 @@
       </c>
       <c r="B775" s="2" t="inlineStr">
         <is>
-          <t>протертые томаты</t>
+          <t>пассата</t>
         </is>
       </c>
       <c r="C775" s="2" t="n">
@@ -32724,7 +32782,7 @@
       </c>
       <c r="H775" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>pureed/protertye tomatoes mapped to passata by user-approved tomato variant policy</t>
         </is>
       </c>
     </row>
@@ -32842,7 +32900,7 @@
       </c>
       <c r="B779" s="2" t="inlineStr">
         <is>
-          <t>винный уксус</t>
+          <t>рисовый уксус</t>
         </is>
       </c>
       <c r="C779" s="2" t="n">
@@ -32864,7 +32922,7 @@
       </c>
       <c r="H779" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>vinegar normalized to rice vinegar; cooking-beverage wording removed</t>
         </is>
       </c>
     </row>
@@ -33000,7 +33058,7 @@
       </c>
       <c r="H783" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>scaled from source; pesto policy approved with explicit grams; large amount high-fat/low-confidence</t>
         </is>
       </c>
     </row>
@@ -33254,7 +33312,7 @@
       </c>
       <c r="B791" s="2" t="inlineStr">
         <is>
-          <t>томатный соус</t>
+          <t>пассата</t>
         </is>
       </c>
       <c r="C791" s="2" t="n">
@@ -33262,7 +33320,7 @@
       </c>
       <c r="D791" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E791" s="2" t="n">
@@ -33270,7 +33328,7 @@
       </c>
       <c r="F791" s="2" t="inlineStr">
         <is>
-          <t>с итальянскими травами</t>
+          <t>tomato sauce normalized to passata + spices policy</t>
         </is>
       </c>
       <c r="G791" s="2" t="inlineStr">
@@ -33280,7 +33338,7 @@
       </c>
       <c r="H791" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>prepared tomato sauce normalized to passata by user-approved tomato sauce policy</t>
         </is>
       </c>
     </row>
@@ -33504,7 +33562,7 @@
       </c>
       <c r="B798" s="2" t="inlineStr">
         <is>
-          <t>куриная колбаска</t>
+          <t>куриное филе</t>
         </is>
       </c>
       <c r="C798" s="2" t="n">
@@ -33520,7 +33578,7 @@
       </c>
       <c r="F798" s="2" t="inlineStr">
         <is>
-          <t>кусочками</t>
+          <t>кусочками, replaces processed poultry product by user decision</t>
         </is>
       </c>
       <c r="G798" s="2" t="inlineStr">
@@ -33530,7 +33588,7 @@
       </c>
       <c r="H798" s="2" t="inlineStr">
         <is>
-          <t>scaled from source; normalized in validated cleanup slice</t>
+          <t>processed poultry product replaced with chicken fillet by user decision</t>
         </is>
       </c>
     </row>
@@ -33542,7 +33600,7 @@
       </c>
       <c r="B799" s="2" t="inlineStr">
         <is>
-          <t>томатный соус аррабиата</t>
+          <t>пассата</t>
         </is>
       </c>
       <c r="C799" s="2" t="n">
@@ -33556,7 +33614,11 @@
       <c r="E799" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="F799" s="2" t="n"/>
+      <c r="F799" s="2" t="inlineStr">
+        <is>
+          <t>arrabbiata normalized to passata + chili/spices policy</t>
+        </is>
+      </c>
       <c r="G799" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -33564,7 +33626,7 @@
       </c>
       <c r="H799" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>prepared arrabbiata sauce normalized to passata by user-approved tomato sauce policy</t>
         </is>
       </c>
     </row>
@@ -33800,7 +33862,7 @@
       </c>
       <c r="B806" s="2" t="inlineStr">
         <is>
-          <t>соль, перец, сахар</t>
+          <t>соль, перец, сахар, чили</t>
         </is>
       </c>
       <c r="C806" s="2" t="inlineStr">
@@ -33820,7 +33882,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H806" s="2" t="n"/>
+      <c r="H806" s="2" t="inlineStr">
+        <is>
+          <t>chili/spices retained for arrabbiata flavor after passata normalization</t>
+        </is>
+      </c>
     </row>
     <row r="807">
       <c r="A807" s="2" t="inlineStr">
@@ -34518,7 +34584,7 @@
       </c>
       <c r="H826" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>chopped/canned tomatoes mapping readiness confirmed by user-approved tomato variant policy</t>
         </is>
       </c>
     </row>
@@ -34716,7 +34782,7 @@
       </c>
       <c r="B832" s="2" t="inlineStr">
         <is>
-          <t>хмели-сунели</t>
+          <t>специи</t>
         </is>
       </c>
       <c r="C832" s="2" t="inlineStr">
@@ -34732,7 +34798,11 @@
       <c r="E832" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F832" s="2" t="n"/>
+      <c r="F832" s="2" t="inlineStr">
+        <is>
+          <t>хмели-сунели</t>
+        </is>
+      </c>
       <c r="G832" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -34740,7 +34810,7 @@
       </c>
       <c r="H832" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>khmeli-suneli mapped to mixed_spices by user decision</t>
         </is>
       </c>
     </row>
@@ -34918,7 +34988,7 @@
       </c>
       <c r="H837" s="2" t="inlineStr">
         <is>
-          <t>from source</t>
+          <t>from source; teriyaki policy approved with modest explicit grams; low-confidence sodium/sugar note acceptable</t>
         </is>
       </c>
     </row>
@@ -37168,7 +37238,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Заправьте майонезом или йогуртом, посолите, поперчите и перемешайте.</t>
+          <t>Заправьте греческим йогуртом, посолите, поперчите и перемешайте.</t>
         </is>
       </c>
     </row>
@@ -38383,7 +38453,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Обжарьте фасоль на смеси масел с чесноком.</t>
+          <t>Обжарьте фасоль и нарезанный тофу на смеси масел с чесноком.</t>
         </is>
       </c>
     </row>
@@ -38413,7 +38483,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Подавайте фасоль с рисом и яйцом или тофу.</t>
+          <t>Подавайте фасоль с тофу и рисом.</t>
         </is>
       </c>
     </row>
@@ -39073,7 +39143,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Посолите, поперчите, добавьте половину хмели-сунели и паприки, перемешайте и оставьте мариноваться на 15—20 минут.</t>
+          <t>Посолите, поперчите, добавьте половину специй и паприки, перемешайте и оставьте мариноваться на 15—20 минут.</t>
         </is>
       </c>
     </row>
@@ -40843,7 +40913,7 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>Замороженный картофель смешайте с приправой для овощей и солью.</t>
+          <t>Замороженный картофель смешайте со специями и солью.</t>
         </is>
       </c>
     </row>
@@ -41398,7 +41468,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Стручковую фасоль отварите 3-4 минуты и остудите.</t>
+          <t>Спаржу отварите 3-4 минуты и остудите.</t>
         </is>
       </c>
     </row>
@@ -41413,7 +41483,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Смешайте капусту, грибы, фасоль, виноград и орехи.</t>
+          <t>Смешайте капусту, грибы, спаржу, виноград и орехи.</t>
         </is>
       </c>
     </row>
@@ -41833,7 +41903,7 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>Добавьте томатный соус, сахар, соль и перец, тушите до густого соуса.</t>
+          <t>Добавьте пассату, сахар, соль и перец, тушите до густого соуса.</t>
         </is>
       </c>
     </row>
@@ -41863,7 +41933,7 @@
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>Колбаски нарежьте наискосок кружочками толщиной примерно 1 см, лук — полукольцами.</t>
+          <t>Куриное филе нарежьте небольшими кусочками, лук — полукольцами.</t>
         </is>
       </c>
     </row>
@@ -41908,7 +41978,7 @@
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>Добавьте оливковое масло, колбаски и нарезанные овощи.</t>
+          <t>Добавьте оливковое масло, куриное филе, лук и сладкий перец.</t>
         </is>
       </c>
     </row>
@@ -41923,7 +41993,7 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>Обжаривайте 2—3 минуты до золотистости, помешивая.</t>
+          <t>Обжаривайте 4-5 минут, затем добавьте пассату, чеснок, соль, перец, сахар и чили; прогрейте до острого томатного соуса.</t>
         </is>
       </c>
     </row>
@@ -41938,7 +42008,7 @@
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>Готовую пасту разложите по тарелкам, украсьте базиликом и тертым сыром и подавайте.</t>
+          <t>Готовую пасту смешайте с соусом, украсьте базиликом и тертым сыром и подавайте.</t>
         </is>
       </c>
     </row>
@@ -42103,7 +42173,7 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>Добавьте говяжий фарш, соль, перец и хмели-сунели, готовьте до изменения цвета.</t>
+          <t>Добавьте говяжий фарш, соль, перец и специи, готовьте до изменения цвета.</t>
         </is>
       </c>
     </row>
@@ -42241,7 +42311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D176"/>
+  <dimension ref="A1:D189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -45255,12 +45325,12 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>Пак-чой и спаржа заменены на пекинскую капусту и стручковую фасоль.</t>
+          <t>Пак-чой заменен на пекинскую капусту; спаржа восстановлена по решению пользователя.</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>Проверить замену при финальной редактуре.</t>
+          <t>Проверить только замену пак-чоя при финальном импорте; спаржу больше не заменять на стручковую фасоль.</t>
         </is>
       </c>
     </row>
@@ -46091,7 +46161,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Решение пользователя применено: голубой сыр заменен на обычный сыр.</t>
+          <t>Решение пользователя применено: сыр с сильным профилем заменен на обычный сыр.</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -46119,6 +46189,292 @@
       <c r="D176" t="inlineStr">
         <is>
           <t>Рецепт переведен в ready; кишмиш не заменялся на изюм.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>intake_032</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Решение пользователя применено: ambiguous dressing normalized to yogurt.</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Крабовые палочки оставлены как generic mapped product; production nutrition rows не добавлялись.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>intake_053</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Решение пользователя применено: ambiguous protein option normalized to tofu.</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Рис оставлен для подачи; тофу отмечен как plant protein anchor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>intake_080</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Решение пользователя применено: product-specific udon wording replaced with generic udon noodles.</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Оставлена staging mapping readiness note; production nutrition row не добавлялся.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>intake_084</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Решение пользователя применено: branded pumpkin wording replaced with generic pumpkin cubes.</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Использована мускатная тыква кубиками как staging-normalized pumpkin; production nutrition row не добавлялся.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>intake_089</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Решение пользователя применено: hummus roll переведен из main в snack/light meal.</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Хумус отмечен как weak plant protein anchor; КБЖУ confidence остается ниже, но это не full main.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>intake_100</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Решение пользователя применено: tomato sauce normalized to passata + spices policy.</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Prepared tomato sauce не оставлен как sugary/oily product; production nutrition row не добавлялся.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>intake_101</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Решение пользователя применено: processed poultry product replaced with chicken fillet.</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Arrabbiata sauce decomposed to passata + spices policy; production nutrition rows не добавлялись.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>intake_098</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Решение пользователя применено: tomato variants normalized; vinegar wording cleaned.</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Cherry tomatoes map to tomato, pureed tomatoes to passata, and vinegar is rice vinegar in staging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>intake_081</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Решение пользователя применено: basmati rice mapping readiness confirmed.</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Ingredient kept as rice with basmati preparation note for staging preview readiness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>intake_086</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Решение пользователя применено: pork chop plural alias and universal seasoning policy confirmed.</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Свиные отбивные нормализованы к singular pork_chop; seasoning treated as mixed_spices/0g.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>intake_096</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Решение пользователя применено: plural egg yolks normalized to egg_yolk mapping.</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Ingredient name set to singular яичный желток for staging preview readiness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>intake_104</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Решение пользователя применено: chopped tomatoes and khmeli-suneli policy confirmed.</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Chopped tomatoes marked mapping-ready; khmeli-suneli normalized to mixed_spices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>intake_062</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Решение пользователя применено: khmeli-suneli normalized to mixed_spices.</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Ingredient name set to специи; хмели-сунели retained only as preparation note.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
recipes: clean final risky intake recipe
</commit_message>
<xml_diff>
--- a/tmp/recipe_intake/cleaned_recipes.xlsx
+++ b/tmp/recipe_intake/cleaned_recipes.xlsx
@@ -6076,7 +6076,7 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Шаурма с фалафелем: основное блюдо на 1 порцию с фалафель замороженный, лаваш «Армянский» тандырный, томаты свежие.</t>
+          <t>Шаурма с фалафелем: основное блюдо на 1 порцию с замороженным фалафелем, лавашем, морковью по-корейски и йогуртово-соевым соусом с лимоном.</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -6110,12 +6110,12 @@
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
-          <t>main, simple, без яиц, без молочки</t>
+          <t>main, simple, без яиц, растительный белок</t>
         </is>
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>Реалистичное фото: шаурма с фалафелем на простой тарелке, видны фалафель замороженный, лаваш «Армянский» тандырный, томаты свежие, морковь по-корейски, огурцы свежие, естественный дневной свет, без текста, логотипов и людей.</t>
+          <t>Реалистичное фото: шаурма с фалафелем на простой тарелке, видны замороженный фалафель, лаваш, томаты, морковь по-корейски, огурцы и легкий йогуртово-соевый соус с лимоном, естественный дневной свет, без текста, логотипов и людей.</t>
         </is>
       </c>
       <c r="M94" s="2" t="inlineStr">
@@ -6870,7 +6870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H847"/>
+  <dimension ref="A1:H849"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -31478,7 +31478,7 @@
       </c>
       <c r="H737" s="2" t="inlineStr">
         <is>
-          <t>frozen/prepared falafel mapping readiness confirmed by user decision; plant protein anchor; frozen/prepared falafel mapping policy approved as generic prepared product; plant protein anchor low-confidence</t>
+          <t>frozen/prepared falafel accepted as generic prepared product; plant protein anchor mapping readiness confirmed</t>
         </is>
       </c>
     </row>
@@ -31580,7 +31580,7 @@
       </c>
       <c r="H740" s="2" t="inlineStr">
         <is>
-          <t>prepared Korean carrot remains low-confidence unless accepted as generic carrot/prepared vegetable</t>
+          <t>Korean carrot accepted as household prepared product; do not decompose into carrot/oil/vinegar/spices; mapping readiness confirmed</t>
         </is>
       </c>
     </row>
@@ -31692,21 +31692,25 @@
       </c>
       <c r="B744" s="2" t="inlineStr">
         <is>
-          <t>соус «Классический майонезный соевый»</t>
+          <t>греческий йогурт</t>
         </is>
       </c>
       <c r="C744" s="2" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="D744" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E744" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="F744" s="2" t="n"/>
+        <v>30</v>
+      </c>
+      <c r="F744" s="2" t="inlineStr">
+        <is>
+          <t>для контролируемого соуса</t>
+        </is>
+      </c>
       <c r="G744" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -31714,23 +31718,23 @@
       </c>
       <c r="H744" s="2" t="inlineStr">
         <is>
-          <t>large prepared mayo-soy sauce remains high-fat/low-confidence; future preview may decompose to generic mayo + soy sauce</t>
+          <t>controlled yogurt-soy-lemon sauce replaces prepared mayo-soy sauce</t>
         </is>
       </c>
     </row>
     <row r="745">
       <c r="A745" s="2" t="inlineStr">
         <is>
-          <t>intake_094</t>
+          <t>intake_093</t>
         </is>
       </c>
       <c r="B745" s="2" t="inlineStr">
         <is>
-          <t>лосось</t>
+          <t>соевый соус</t>
         </is>
       </c>
       <c r="C745" s="2" t="n">
-        <v>200</v>
+        <v>5</v>
       </c>
       <c r="D745" s="2" t="inlineStr">
         <is>
@@ -31738,33 +31742,37 @@
         </is>
       </c>
       <c r="E745" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="F745" s="2" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="F745" s="2" t="inlineStr">
+        <is>
+          <t>для контролируемого соуса</t>
+        </is>
+      </c>
       <c r="G745" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H745" s="2" t="inlineStr">
         <is>
-          <t>normalized in validated cleanup slice</t>
+          <t>soy sauce kept as accepted standard condiment with explicit grams</t>
         </is>
       </c>
     </row>
     <row r="746">
       <c r="A746" s="2" t="inlineStr">
         <is>
-          <t>intake_094</t>
+          <t>intake_093</t>
         </is>
       </c>
       <c r="B746" s="2" t="inlineStr">
         <is>
-          <t>шпинат свежий</t>
+          <t>лимонный сок</t>
         </is>
       </c>
       <c r="C746" s="2" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="D746" s="2" t="inlineStr">
         <is>
@@ -31772,15 +31780,23 @@
         </is>
       </c>
       <c r="E746" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="F746" s="2" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="F746" s="2" t="inlineStr">
+        <is>
+          <t>для контролируемого соуса</t>
+        </is>
+      </c>
       <c r="G746" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H746" s="2" t="n"/>
+      <c r="H746" s="2" t="inlineStr">
+        <is>
+          <t>normalized citrus juice for controlled sauce</t>
+        </is>
+      </c>
     </row>
     <row r="747">
       <c r="A747" s="2" t="inlineStr">
@@ -31790,11 +31806,11 @@
       </c>
       <c r="B747" s="2" t="inlineStr">
         <is>
-          <t>сливки</t>
+          <t>лосось</t>
         </is>
       </c>
       <c r="C747" s="2" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="D747" s="2" t="inlineStr">
         <is>
@@ -31802,12 +31818,12 @@
         </is>
       </c>
       <c r="E747" s="2" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="F747" s="2" t="n"/>
       <c r="G747" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H747" s="2" t="inlineStr">
@@ -31824,21 +31840,19 @@
       </c>
       <c r="B748" s="2" t="inlineStr">
         <is>
-          <t>чеснок</t>
-        </is>
-      </c>
-      <c r="C748" s="2" t="inlineStr">
-        <is>
-          <t>1/4</t>
-        </is>
+          <t>шпинат свежий</t>
+        </is>
+      </c>
+      <c r="C748" s="2" t="n">
+        <v>25</v>
       </c>
       <c r="D748" s="2" t="inlineStr">
         <is>
-          <t>зубчик</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E748" s="2" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="F748" s="2" t="n"/>
       <c r="G748" s="2" t="inlineStr">
@@ -31856,11 +31870,11 @@
       </c>
       <c r="B749" s="2" t="inlineStr">
         <is>
-          <t>сыр гауда</t>
+          <t>сливки</t>
         </is>
       </c>
       <c r="C749" s="2" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D749" s="2" t="inlineStr">
         <is>
@@ -31868,7 +31882,7 @@
         </is>
       </c>
       <c r="E749" s="2" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="F749" s="2" t="n"/>
       <c r="G749" s="2" t="inlineStr">
@@ -31878,7 +31892,7 @@
       </c>
       <c r="H749" s="2" t="inlineStr">
         <is>
-          <t>strong cheese variant replaced with gouda by user decision</t>
+          <t>normalized in validated cleanup slice</t>
         </is>
       </c>
     </row>
@@ -31890,19 +31904,21 @@
       </c>
       <c r="B750" s="2" t="inlineStr">
         <is>
-          <t>кедровые орехи</t>
-        </is>
-      </c>
-      <c r="C750" s="2" t="n">
-        <v>5</v>
+          <t>чеснок</t>
+        </is>
+      </c>
+      <c r="C750" s="2" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
       </c>
       <c r="D750" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>зубчик</t>
         </is>
       </c>
       <c r="E750" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F750" s="2" t="n"/>
       <c r="G750" s="2" t="inlineStr">
@@ -31915,16 +31931,16 @@
     <row r="751">
       <c r="A751" s="2" t="inlineStr">
         <is>
-          <t>intake_095</t>
+          <t>intake_094</t>
         </is>
       </c>
       <c r="B751" s="2" t="inlineStr">
         <is>
-          <t>пекинская капуста</t>
+          <t>сыр гауда</t>
         </is>
       </c>
       <c r="C751" s="2" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D751" s="2" t="inlineStr">
         <is>
@@ -31932,13 +31948,9 @@
         </is>
       </c>
       <c r="E751" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="F751" s="2" t="inlineStr">
-        <is>
-          <t>вместо пак-чоя</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="F751" s="2" t="n"/>
       <c r="G751" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -31946,23 +31958,23 @@
       </c>
       <c r="H751" s="2" t="inlineStr">
         <is>
-          <t>accessible replacement</t>
+          <t>strong cheese variant replaced with gouda by user decision</t>
         </is>
       </c>
     </row>
     <row r="752">
       <c r="A752" s="2" t="inlineStr">
         <is>
-          <t>intake_095</t>
+          <t>intake_094</t>
         </is>
       </c>
       <c r="B752" s="2" t="inlineStr">
         <is>
-          <t>шампиньоны</t>
+          <t>кедровые орехи</t>
         </is>
       </c>
       <c r="C752" s="2" t="n">
-        <v>80</v>
+        <v>5</v>
       </c>
       <c r="D752" s="2" t="inlineStr">
         <is>
@@ -31970,23 +31982,15 @@
         </is>
       </c>
       <c r="E752" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="F752" s="2" t="inlineStr">
-        <is>
-          <t>ломтиками</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="F752" s="2" t="n"/>
       <c r="G752" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H752" s="2" t="inlineStr">
-        <is>
-          <t>amount inferred</t>
-        </is>
-      </c>
+      <c r="H752" s="2" t="n"/>
     </row>
     <row r="753">
       <c r="A753" s="2" t="inlineStr">
@@ -31996,11 +32000,11 @@
       </c>
       <c r="B753" s="2" t="inlineStr">
         <is>
-          <t>спаржа</t>
+          <t>пекинская капуста</t>
         </is>
       </c>
       <c r="C753" s="2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="D753" s="2" t="inlineStr">
         <is>
@@ -32008,11 +32012,11 @@
         </is>
       </c>
       <c r="E753" s="2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F753" s="2" t="inlineStr">
         <is>
-          <t>восстановлено вместо green beans</t>
+          <t>вместо пак-чоя</t>
         </is>
       </c>
       <c r="G753" s="2" t="inlineStr">
@@ -32022,7 +32026,7 @@
       </c>
       <c r="H753" s="2" t="inlineStr">
         <is>
-          <t>asparagus restored by user decision; asparagus mapping readiness confirmed</t>
+          <t>accessible replacement</t>
         </is>
       </c>
     </row>
@@ -32034,11 +32038,11 @@
       </c>
       <c r="B754" s="2" t="inlineStr">
         <is>
-          <t>виноград кишмиш</t>
+          <t>шампиньоны</t>
         </is>
       </c>
       <c r="C754" s="2" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="D754" s="2" t="inlineStr">
         <is>
@@ -32046,9 +32050,13 @@
         </is>
       </c>
       <c r="E754" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="F754" s="2" t="n"/>
+        <v>80</v>
+      </c>
+      <c r="F754" s="2" t="inlineStr">
+        <is>
+          <t>ломтиками</t>
+        </is>
+      </c>
       <c r="G754" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -32056,7 +32064,7 @@
       </c>
       <c r="H754" s="2" t="inlineStr">
         <is>
-          <t>from source; fresh kishmish grape mapping confirmed by user decision; fresh grape/kishmish mapping readiness confirmed; avoid beverage-alias substring matching</t>
+          <t>amount inferred</t>
         </is>
       </c>
     </row>
@@ -32068,11 +32076,11 @@
       </c>
       <c r="B755" s="2" t="inlineStr">
         <is>
-          <t>грецкие орехи</t>
+          <t>спаржа</t>
         </is>
       </c>
       <c r="C755" s="2" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="D755" s="2" t="inlineStr">
         <is>
@@ -32080,11 +32088,11 @@
         </is>
       </c>
       <c r="E755" s="2" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="F755" s="2" t="inlineStr">
         <is>
-          <t>рубленые</t>
+          <t>восстановлено вместо green beans</t>
         </is>
       </c>
       <c r="G755" s="2" t="inlineStr">
@@ -32094,7 +32102,7 @@
       </c>
       <c r="H755" s="2" t="inlineStr">
         <is>
-          <t>amount inferred</t>
+          <t>asparagus restored by user decision; asparagus mapping readiness confirmed</t>
         </is>
       </c>
     </row>
@@ -32106,11 +32114,11 @@
       </c>
       <c r="B756" s="2" t="inlineStr">
         <is>
-          <t>миндаль</t>
+          <t>виноград кишмиш</t>
         </is>
       </c>
       <c r="C756" s="2" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D756" s="2" t="inlineStr">
         <is>
@@ -32118,13 +32126,9 @@
         </is>
       </c>
       <c r="E756" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F756" s="2" t="inlineStr">
-        <is>
-          <t>рубленый</t>
-        </is>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="F756" s="2" t="n"/>
       <c r="G756" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -32132,7 +32136,7 @@
       </c>
       <c r="H756" s="2" t="inlineStr">
         <is>
-          <t>amount inferred</t>
+          <t>from source; fresh kishmish grape mapping confirmed by user decision; fresh grape/kishmish mapping readiness confirmed; avoid beverage-alias substring matching</t>
         </is>
       </c>
     </row>
@@ -32144,21 +32148,25 @@
       </c>
       <c r="B757" s="2" t="inlineStr">
         <is>
-          <t>оливковое масло</t>
+          <t>грецкие орехи</t>
         </is>
       </c>
       <c r="C757" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D757" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E757" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F757" s="2" t="n"/>
+        <v>10</v>
+      </c>
+      <c r="F757" s="2" t="inlineStr">
+        <is>
+          <t>рубленые</t>
+        </is>
+      </c>
       <c r="G757" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -32166,7 +32174,7 @@
       </c>
       <c r="H757" s="2" t="inlineStr">
         <is>
-          <t>from source</t>
+          <t>amount inferred</t>
         </is>
       </c>
     </row>
@@ -32178,21 +32186,25 @@
       </c>
       <c r="B758" s="2" t="inlineStr">
         <is>
-          <t>апельсиновый сок</t>
+          <t>миндаль</t>
         </is>
       </c>
       <c r="C758" s="2" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="D758" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E758" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="F758" s="2" t="n"/>
+        <v>10</v>
+      </c>
+      <c r="F758" s="2" t="inlineStr">
+        <is>
+          <t>рубленый</t>
+        </is>
+      </c>
       <c r="G758" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -32200,7 +32212,7 @@
       </c>
       <c r="H758" s="2" t="inlineStr">
         <is>
-          <t>from source</t>
+          <t>amount inferred</t>
         </is>
       </c>
     </row>
@@ -32212,49 +32224,53 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>соль</t>
-        </is>
-      </c>
-      <c r="C759" s="2" t="inlineStr">
-        <is>
-          <t>по вкусу</t>
-        </is>
+          <t>оливковое масло</t>
+        </is>
+      </c>
+      <c r="C759" s="2" t="n">
+        <v>15</v>
       </c>
       <c r="D759" s="2" t="inlineStr">
         <is>
-          <t>по вкусу</t>
-        </is>
-      </c>
-      <c r="E759" s="2" t="n"/>
+          <t>мл</t>
+        </is>
+      </c>
+      <c r="E759" s="2" t="n">
+        <v>15</v>
+      </c>
       <c r="F759" s="2" t="n"/>
       <c r="G759" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H759" s="2" t="n"/>
+      <c r="H759" s="2" t="inlineStr">
+        <is>
+          <t>from source</t>
+        </is>
+      </c>
     </row>
     <row r="760">
       <c r="A760" s="2" t="inlineStr">
         <is>
-          <t>intake_096</t>
+          <t>intake_095</t>
         </is>
       </c>
       <c r="B760" s="2" t="inlineStr">
         <is>
-          <t>спагетти</t>
+          <t>апельсиновый сок</t>
         </is>
       </c>
       <c r="C760" s="2" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="D760" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>мл</t>
         </is>
       </c>
       <c r="E760" s="2" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="F760" s="2" t="n"/>
       <c r="G760" s="2" t="inlineStr">
@@ -32271,40 +32287,32 @@
     <row r="761">
       <c r="A761" s="2" t="inlineStr">
         <is>
-          <t>intake_096</t>
+          <t>intake_095</t>
         </is>
       </c>
       <c r="B761" s="2" t="inlineStr">
         <is>
-          <t>сливки 20%</t>
-        </is>
-      </c>
-      <c r="C761" s="2" t="n">
-        <v>80</v>
+          <t>соль</t>
+        </is>
+      </c>
+      <c r="C761" s="2" t="inlineStr">
+        <is>
+          <t>по вкусу</t>
+        </is>
       </c>
       <c r="D761" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
-        </is>
-      </c>
-      <c r="E761" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="F761" s="2" t="inlineStr">
-        <is>
-          <t>для соуса</t>
-        </is>
-      </c>
+          <t>по вкусу</t>
+        </is>
+      </c>
+      <c r="E761" s="2" t="n"/>
+      <c r="F761" s="2" t="n"/>
       <c r="G761" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H761" s="2" t="inlineStr">
-        <is>
-          <t>from source</t>
-        </is>
-      </c>
+      <c r="H761" s="2" t="n"/>
     </row>
     <row r="762">
       <c r="A762" s="2" t="inlineStr">
@@ -32314,11 +32322,11 @@
       </c>
       <c r="B762" s="2" t="inlineStr">
         <is>
-          <t>бекон сырокопченый</t>
+          <t>спагетти</t>
         </is>
       </c>
       <c r="C762" s="2" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="D762" s="2" t="inlineStr">
         <is>
@@ -32326,16 +32334,12 @@
         </is>
       </c>
       <c r="E762" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="F762" s="2" t="inlineStr">
-        <is>
-          <t>кусочками</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="F762" s="2" t="n"/>
       <c r="G762" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H762" s="2" t="inlineStr">
@@ -32352,28 +32356,28 @@
       </c>
       <c r="B763" s="2" t="inlineStr">
         <is>
-          <t>пармезан</t>
+          <t>сливки 20%</t>
         </is>
       </c>
       <c r="C763" s="2" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="D763" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>мл</t>
         </is>
       </c>
       <c r="E763" s="2" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="F763" s="2" t="inlineStr">
         <is>
-          <t>для подачи</t>
+          <t>для соуса</t>
         </is>
       </c>
       <c r="G763" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H763" s="2" t="inlineStr">
@@ -32390,21 +32394,25 @@
       </c>
       <c r="B764" s="2" t="inlineStr">
         <is>
-          <t>яичный желток</t>
+          <t>бекон сырокопченый</t>
         </is>
       </c>
       <c r="C764" s="2" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="D764" s="2" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E764" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="F764" s="2" t="n"/>
+        <v>60</v>
+      </c>
+      <c r="F764" s="2" t="inlineStr">
+        <is>
+          <t>кусочками</t>
+        </is>
+      </c>
       <c r="G764" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -32412,7 +32420,7 @@
       </c>
       <c r="H764" s="2" t="inlineStr">
         <is>
-          <t>plural egg yolks mapped to egg_yolk by user decision</t>
+          <t>from source</t>
         </is>
       </c>
     </row>
@@ -32424,27 +32432,35 @@
       </c>
       <c r="B765" s="2" t="inlineStr">
         <is>
-          <t>мускатный орех</t>
-        </is>
-      </c>
-      <c r="C765" s="2" t="inlineStr">
-        <is>
-          <t>по вкусу</t>
-        </is>
+          <t>пармезан</t>
+        </is>
+      </c>
+      <c r="C765" s="2" t="n">
+        <v>20</v>
       </c>
       <c r="D765" s="2" t="inlineStr">
         <is>
-          <t>по вкусу</t>
-        </is>
-      </c>
-      <c r="E765" s="2" t="n"/>
-      <c r="F765" s="2" t="n"/>
+          <t>г</t>
+        </is>
+      </c>
+      <c r="E765" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F765" s="2" t="inlineStr">
+        <is>
+          <t>для подачи</t>
+        </is>
+      </c>
       <c r="G765" s="2" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H765" s="2" t="n"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H765" s="2" t="inlineStr">
+        <is>
+          <t>from source</t>
+        </is>
+      </c>
     </row>
     <row r="766">
       <c r="A766" s="2" t="inlineStr">
@@ -32454,27 +32470,31 @@
       </c>
       <c r="B766" s="2" t="inlineStr">
         <is>
-          <t>перец</t>
-        </is>
-      </c>
-      <c r="C766" s="2" t="inlineStr">
-        <is>
-          <t>по вкусу</t>
-        </is>
+          <t>яичный желток</t>
+        </is>
+      </c>
+      <c r="C766" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D766" s="2" t="inlineStr">
         <is>
-          <t>по вкусу</t>
-        </is>
-      </c>
-      <c r="E766" s="2" t="n"/>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E766" s="2" t="n">
+        <v>18</v>
+      </c>
       <c r="F766" s="2" t="n"/>
       <c r="G766" s="2" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H766" s="2" t="n"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H766" s="2" t="inlineStr">
+        <is>
+          <t>plural egg yolks mapped to egg_yolk by user decision</t>
+        </is>
+      </c>
     </row>
     <row r="767">
       <c r="A767" s="2" t="inlineStr">
@@ -32484,7 +32504,7 @@
       </c>
       <c r="B767" s="2" t="inlineStr">
         <is>
-          <t>соль</t>
+          <t>мускатный орех</t>
         </is>
       </c>
       <c r="C767" s="2" t="inlineStr">
@@ -32509,74 +32529,62 @@
     <row r="768">
       <c r="A768" s="2" t="inlineStr">
         <is>
-          <t>intake_097</t>
+          <t>intake_096</t>
         </is>
       </c>
       <c r="B768" s="2" t="inlineStr">
         <is>
-          <t>спагетти</t>
-        </is>
-      </c>
-      <c r="C768" s="2" t="n">
-        <v>90</v>
+          <t>перец</t>
+        </is>
+      </c>
+      <c r="C768" s="2" t="inlineStr">
+        <is>
+          <t>по вкусу</t>
+        </is>
       </c>
       <c r="D768" s="2" t="inlineStr">
         <is>
-          <t>г</t>
-        </is>
-      </c>
-      <c r="E768" s="2" t="n">
-        <v>90</v>
-      </c>
+          <t>по вкусу</t>
+        </is>
+      </c>
+      <c r="E768" s="2" t="n"/>
       <c r="F768" s="2" t="n"/>
       <c r="G768" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H768" s="2" t="inlineStr">
-        <is>
-          <t>scaled from source</t>
-        </is>
-      </c>
+      <c r="H768" s="2" t="n"/>
     </row>
     <row r="769">
       <c r="A769" s="2" t="inlineStr">
         <is>
-          <t>intake_097</t>
+          <t>intake_096</t>
         </is>
       </c>
       <c r="B769" s="2" t="inlineStr">
         <is>
-          <t>пармезан</t>
-        </is>
-      </c>
-      <c r="C769" s="2" t="n">
-        <v>15</v>
+          <t>соль</t>
+        </is>
+      </c>
+      <c r="C769" s="2" t="inlineStr">
+        <is>
+          <t>по вкусу</t>
+        </is>
       </c>
       <c r="D769" s="2" t="inlineStr">
         <is>
-          <t>г</t>
-        </is>
-      </c>
-      <c r="E769" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F769" s="2" t="inlineStr">
-        <is>
-          <t>мелко натереть</t>
-        </is>
-      </c>
+          <t>по вкусу</t>
+        </is>
+      </c>
+      <c r="E769" s="2" t="n"/>
+      <c r="F769" s="2" t="n"/>
       <c r="G769" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H769" s="2" t="inlineStr">
-        <is>
-          <t>scaled from source</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H769" s="2" t="n"/>
     </row>
     <row r="770">
       <c r="A770" s="2" t="inlineStr">
@@ -32586,19 +32594,19 @@
       </c>
       <c r="B770" s="2" t="inlineStr">
         <is>
-          <t>оливковое масло</t>
+          <t>спагетти</t>
         </is>
       </c>
       <c r="C770" s="2" t="n">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="D770" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E770" s="2" t="n">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="F770" s="2" t="n"/>
       <c r="G770" s="2" t="inlineStr">
@@ -32620,11 +32628,11 @@
       </c>
       <c r="B771" s="2" t="inlineStr">
         <is>
-          <t>черный перец</t>
+          <t>пармезан</t>
         </is>
       </c>
       <c r="C771" s="2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D771" s="2" t="inlineStr">
         <is>
@@ -32632,16 +32640,16 @@
         </is>
       </c>
       <c r="E771" s="2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F771" s="2" t="inlineStr">
         <is>
-          <t>свежемолотый</t>
+          <t>мелко натереть</t>
         </is>
       </c>
       <c r="G771" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H771" s="2" t="inlineStr">
@@ -32658,41 +32666,45 @@
       </c>
       <c r="B772" s="2" t="inlineStr">
         <is>
-          <t>соль</t>
-        </is>
-      </c>
-      <c r="C772" s="2" t="inlineStr">
-        <is>
-          <t>по вкусу</t>
-        </is>
+          <t>оливковое масло</t>
+        </is>
+      </c>
+      <c r="C772" s="2" t="n">
+        <v>12</v>
       </c>
       <c r="D772" s="2" t="inlineStr">
         <is>
-          <t>по вкусу</t>
-        </is>
-      </c>
-      <c r="E772" s="2" t="n"/>
+          <t>мл</t>
+        </is>
+      </c>
+      <c r="E772" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="F772" s="2" t="n"/>
       <c r="G772" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H772" s="2" t="n"/>
+      <c r="H772" s="2" t="inlineStr">
+        <is>
+          <t>scaled from source</t>
+        </is>
+      </c>
     </row>
     <row r="773">
       <c r="A773" s="2" t="inlineStr">
         <is>
-          <t>intake_098</t>
+          <t>intake_097</t>
         </is>
       </c>
       <c r="B773" s="2" t="inlineStr">
         <is>
-          <t>паста</t>
+          <t>черный перец</t>
         </is>
       </c>
       <c r="C773" s="2" t="n">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="D773" s="2" t="inlineStr">
         <is>
@@ -32700,9 +32712,13 @@
         </is>
       </c>
       <c r="E773" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="F773" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="F773" s="2" t="inlineStr">
+        <is>
+          <t>свежемолотый</t>
+        </is>
+      </c>
       <c r="G773" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -32717,40 +32733,32 @@
     <row r="774">
       <c r="A774" s="2" t="inlineStr">
         <is>
-          <t>intake_098</t>
+          <t>intake_097</t>
         </is>
       </c>
       <c r="B774" s="2" t="inlineStr">
         <is>
-          <t>помидоры черри</t>
-        </is>
-      </c>
-      <c r="C774" s="2" t="n">
-        <v>75</v>
+          <t>соль</t>
+        </is>
+      </c>
+      <c r="C774" s="2" t="inlineStr">
+        <is>
+          <t>по вкусу</t>
+        </is>
       </c>
       <c r="D774" s="2" t="inlineStr">
         <is>
-          <t>г</t>
-        </is>
-      </c>
-      <c r="E774" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="F774" s="2" t="inlineStr">
-        <is>
-          <t>половинками; maps to tomato policy</t>
-        </is>
-      </c>
+          <t>по вкусу</t>
+        </is>
+      </c>
+      <c r="E774" s="2" t="n"/>
+      <c r="F774" s="2" t="n"/>
       <c r="G774" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H774" s="2" t="inlineStr">
-        <is>
-          <t>cherry tomatoes mapped to tomato by user-approved tomato variant policy</t>
-        </is>
-      </c>
+      <c r="H774" s="2" t="n"/>
     </row>
     <row r="775">
       <c r="A775" s="2" t="inlineStr">
@@ -32760,11 +32768,11 @@
       </c>
       <c r="B775" s="2" t="inlineStr">
         <is>
-          <t>пассата</t>
+          <t>паста</t>
         </is>
       </c>
       <c r="C775" s="2" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D775" s="2" t="inlineStr">
         <is>
@@ -32772,7 +32780,7 @@
         </is>
       </c>
       <c r="E775" s="2" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F775" s="2" t="n"/>
       <c r="G775" s="2" t="inlineStr">
@@ -32782,7 +32790,7 @@
       </c>
       <c r="H775" s="2" t="inlineStr">
         <is>
-          <t>pureed/protertye tomatoes mapped to passata by user-approved tomato variant policy</t>
+          <t>scaled from source</t>
         </is>
       </c>
     </row>
@@ -32794,11 +32802,11 @@
       </c>
       <c r="B776" s="2" t="inlineStr">
         <is>
-          <t>тунец консервированный</t>
+          <t>помидоры черри</t>
         </is>
       </c>
       <c r="C776" s="2" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="D776" s="2" t="inlineStr">
         <is>
@@ -32806,21 +32814,21 @@
         </is>
       </c>
       <c r="E776" s="2" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="F776" s="2" t="inlineStr">
         <is>
-          <t>без жидкости</t>
+          <t>половинками; maps to tomato policy</t>
         </is>
       </c>
       <c r="G776" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H776" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>cherry tomatoes mapped to tomato by user-approved tomato variant policy</t>
         </is>
       </c>
     </row>
@@ -32832,19 +32840,19 @@
       </c>
       <c r="B777" s="2" t="inlineStr">
         <is>
-          <t>оливковое масло</t>
+          <t>пассата</t>
         </is>
       </c>
       <c r="C777" s="2" t="n">
-        <v>8</v>
+        <v>75</v>
       </c>
       <c r="D777" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E777" s="2" t="n">
-        <v>8</v>
+        <v>75</v>
       </c>
       <c r="F777" s="2" t="n"/>
       <c r="G777" s="2" t="inlineStr">
@@ -32854,7 +32862,7 @@
       </c>
       <c r="H777" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>pureed/protertye tomatoes mapped to passata by user-approved tomato variant policy</t>
         </is>
       </c>
     </row>
@@ -32866,11 +32874,11 @@
       </c>
       <c r="B778" s="2" t="inlineStr">
         <is>
-          <t>сливочный сыр</t>
+          <t>тунец консервированный</t>
         </is>
       </c>
       <c r="C778" s="2" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="D778" s="2" t="inlineStr">
         <is>
@@ -32878,12 +32886,16 @@
         </is>
       </c>
       <c r="E778" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F778" s="2" t="n"/>
+        <v>50</v>
+      </c>
+      <c r="F778" s="2" t="inlineStr">
+        <is>
+          <t>без жидкости</t>
+        </is>
+      </c>
       <c r="G778" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H778" s="2" t="inlineStr">
@@ -32900,11 +32912,11 @@
       </c>
       <c r="B779" s="2" t="inlineStr">
         <is>
-          <t>рисовый уксус</t>
+          <t>оливковое масло</t>
         </is>
       </c>
       <c r="C779" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D779" s="2" t="inlineStr">
         <is>
@@ -32912,7 +32924,7 @@
         </is>
       </c>
       <c r="E779" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F779" s="2" t="n"/>
       <c r="G779" s="2" t="inlineStr">
@@ -32922,7 +32934,7 @@
       </c>
       <c r="H779" s="2" t="inlineStr">
         <is>
-          <t>vinegar normalized to rice vinegar; cooking-beverage wording removed</t>
+          <t>scaled from source</t>
         </is>
       </c>
     </row>
@@ -32934,49 +32946,53 @@
       </c>
       <c r="B780" s="2" t="inlineStr">
         <is>
-          <t>соль, сахар, чили</t>
-        </is>
-      </c>
-      <c r="C780" s="2" t="inlineStr">
-        <is>
-          <t>по вкусу</t>
-        </is>
+          <t>сливочный сыр</t>
+        </is>
+      </c>
+      <c r="C780" s="2" t="n">
+        <v>10</v>
       </c>
       <c r="D780" s="2" t="inlineStr">
         <is>
-          <t>по вкусу</t>
-        </is>
-      </c>
-      <c r="E780" s="2" t="n"/>
+          <t>г</t>
+        </is>
+      </c>
+      <c r="E780" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="F780" s="2" t="n"/>
       <c r="G780" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H780" s="2" t="n"/>
+      <c r="H780" s="2" t="inlineStr">
+        <is>
+          <t>scaled from source</t>
+        </is>
+      </c>
     </row>
     <row r="781">
       <c r="A781" s="2" t="inlineStr">
         <is>
-          <t>intake_099</t>
+          <t>intake_098</t>
         </is>
       </c>
       <c r="B781" s="2" t="inlineStr">
         <is>
-          <t>длинная паста</t>
+          <t>рисовый уксус</t>
         </is>
       </c>
       <c r="C781" s="2" t="n">
-        <v>80</v>
+        <v>5</v>
       </c>
       <c r="D781" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>мл</t>
         </is>
       </c>
       <c r="E781" s="2" t="n">
-        <v>80</v>
+        <v>5</v>
       </c>
       <c r="F781" s="2" t="n"/>
       <c r="G781" s="2" t="inlineStr">
@@ -32986,47 +33002,39 @@
       </c>
       <c r="H781" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>vinegar normalized to rice vinegar; cooking-beverage wording removed</t>
         </is>
       </c>
     </row>
     <row r="782">
       <c r="A782" s="2" t="inlineStr">
         <is>
-          <t>intake_099</t>
+          <t>intake_098</t>
         </is>
       </c>
       <c r="B782" s="2" t="inlineStr">
         <is>
-          <t>креветки</t>
-        </is>
-      </c>
-      <c r="C782" s="2" t="n">
-        <v>80</v>
+          <t>соль, сахар, чили</t>
+        </is>
+      </c>
+      <c r="C782" s="2" t="inlineStr">
+        <is>
+          <t>по вкусу</t>
+        </is>
       </c>
       <c r="D782" s="2" t="inlineStr">
         <is>
-          <t>г</t>
-        </is>
-      </c>
-      <c r="E782" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="F782" s="2" t="inlineStr">
-        <is>
-          <t>очищенные</t>
-        </is>
-      </c>
+          <t>по вкусу</t>
+        </is>
+      </c>
+      <c r="E782" s="2" t="n"/>
+      <c r="F782" s="2" t="n"/>
       <c r="G782" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H782" s="2" t="inlineStr">
-        <is>
-          <t>scaled from source; normalized in validated cleanup slice</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H782" s="2" t="n"/>
     </row>
     <row r="783">
       <c r="A783" s="2" t="inlineStr">
@@ -33036,11 +33044,11 @@
       </c>
       <c r="B783" s="2" t="inlineStr">
         <is>
-          <t>песто</t>
+          <t>длинная паста</t>
         </is>
       </c>
       <c r="C783" s="2" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="D783" s="2" t="inlineStr">
         <is>
@@ -33048,7 +33056,7 @@
         </is>
       </c>
       <c r="E783" s="2" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F783" s="2" t="n"/>
       <c r="G783" s="2" t="inlineStr">
@@ -33058,7 +33066,7 @@
       </c>
       <c r="H783" s="2" t="inlineStr">
         <is>
-          <t>scaled from source; pesto policy approved with explicit grams; large amount high-fat/low-confidence</t>
+          <t>scaled from source</t>
         </is>
       </c>
     </row>
@@ -33070,11 +33078,11 @@
       </c>
       <c r="B784" s="2" t="inlineStr">
         <is>
-          <t>пармезан</t>
+          <t>креветки</t>
         </is>
       </c>
       <c r="C784" s="2" t="n">
-        <v>15</v>
+        <v>80</v>
       </c>
       <c r="D784" s="2" t="inlineStr">
         <is>
@@ -33082,9 +33090,13 @@
         </is>
       </c>
       <c r="E784" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F784" s="2" t="n"/>
+        <v>80</v>
+      </c>
+      <c r="F784" s="2" t="inlineStr">
+        <is>
+          <t>очищенные</t>
+        </is>
+      </c>
       <c r="G784" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -33092,7 +33104,7 @@
       </c>
       <c r="H784" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>scaled from source; normalized in validated cleanup slice</t>
         </is>
       </c>
     </row>
@@ -33104,19 +33116,19 @@
       </c>
       <c r="B785" s="2" t="inlineStr">
         <is>
-          <t>сливки 20%</t>
+          <t>песто</t>
         </is>
       </c>
       <c r="C785" s="2" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="D785" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E785" s="2" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="F785" s="2" t="n"/>
       <c r="G785" s="2" t="inlineStr">
@@ -33126,7 +33138,7 @@
       </c>
       <c r="H785" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>scaled from source; pesto policy approved with explicit grams; large amount high-fat/low-confidence</t>
         </is>
       </c>
     </row>
@@ -33138,28 +33150,24 @@
       </c>
       <c r="B786" s="2" t="inlineStr">
         <is>
-          <t>чеснок</t>
+          <t>пармезан</t>
         </is>
       </c>
       <c r="C786" s="2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D786" s="2" t="inlineStr">
         <is>
-          <t>зубчик</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E786" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F786" s="2" t="inlineStr">
-        <is>
-          <t>измельчить</t>
-        </is>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F786" s="2" t="n"/>
       <c r="G786" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H786" s="2" t="inlineStr">
@@ -33176,11 +33184,11 @@
       </c>
       <c r="B787" s="2" t="inlineStr">
         <is>
-          <t>оливковое масло</t>
+          <t>сливки 20%</t>
         </is>
       </c>
       <c r="C787" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D787" s="2" t="inlineStr">
         <is>
@@ -33188,7 +33196,7 @@
         </is>
       </c>
       <c r="E787" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F787" s="2" t="n"/>
       <c r="G787" s="2" t="inlineStr">
@@ -33210,7 +33218,7 @@
       </c>
       <c r="B788" s="2" t="inlineStr">
         <is>
-          <t>перец чили</t>
+          <t>чеснок</t>
         </is>
       </c>
       <c r="C788" s="2" t="n">
@@ -33218,13 +33226,17 @@
       </c>
       <c r="D788" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>зубчик</t>
         </is>
       </c>
       <c r="E788" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F788" s="2" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="F788" s="2" t="inlineStr">
+        <is>
+          <t>измельчить</t>
+        </is>
+      </c>
       <c r="G788" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -33232,31 +33244,31 @@
       </c>
       <c r="H788" s="2" t="inlineStr">
         <is>
-          <t>normalized in validated cleanup slice</t>
+          <t>scaled from source</t>
         </is>
       </c>
     </row>
     <row r="789">
       <c r="A789" s="2" t="inlineStr">
         <is>
-          <t>intake_100</t>
+          <t>intake_099</t>
         </is>
       </c>
       <c r="B789" s="2" t="inlineStr">
         <is>
-          <t>цельнозерновая паста</t>
+          <t>оливковое масло</t>
         </is>
       </c>
       <c r="C789" s="2" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="D789" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>мл</t>
         </is>
       </c>
       <c r="E789" s="2" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="F789" s="2" t="n"/>
       <c r="G789" s="2" t="inlineStr">
@@ -33266,23 +33278,23 @@
       </c>
       <c r="H789" s="2" t="inlineStr">
         <is>
-          <t>scaled from source; normalized in validated cleanup slice</t>
+          <t>scaled from source</t>
         </is>
       </c>
     </row>
     <row r="790">
       <c r="A790" s="2" t="inlineStr">
         <is>
-          <t>intake_100</t>
+          <t>intake_099</t>
         </is>
       </c>
       <c r="B790" s="2" t="inlineStr">
         <is>
-          <t>говяжий фарш</t>
+          <t>перец чили</t>
         </is>
       </c>
       <c r="C790" s="2" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="D790" s="2" t="inlineStr">
         <is>
@@ -33290,17 +33302,17 @@
         </is>
       </c>
       <c r="E790" s="2" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F790" s="2" t="n"/>
       <c r="G790" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H790" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>normalized in validated cleanup slice</t>
         </is>
       </c>
     </row>
@@ -33312,11 +33324,11 @@
       </c>
       <c r="B791" s="2" t="inlineStr">
         <is>
-          <t>пассата</t>
+          <t>цельнозерновая паста</t>
         </is>
       </c>
       <c r="C791" s="2" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="D791" s="2" t="inlineStr">
         <is>
@@ -33324,13 +33336,9 @@
         </is>
       </c>
       <c r="E791" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="F791" s="2" t="inlineStr">
-        <is>
-          <t>tomato sauce normalized to passata + spices policy</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="F791" s="2" t="n"/>
       <c r="G791" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -33338,7 +33346,7 @@
       </c>
       <c r="H791" s="2" t="inlineStr">
         <is>
-          <t>prepared tomato sauce normalized to passata by user-approved tomato sauce policy</t>
+          <t>scaled from source; normalized in validated cleanup slice</t>
         </is>
       </c>
     </row>
@@ -33350,28 +33358,24 @@
       </c>
       <c r="B792" s="2" t="inlineStr">
         <is>
-          <t>чеснок</t>
+          <t>говяжий фарш</t>
         </is>
       </c>
       <c r="C792" s="2" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="D792" s="2" t="inlineStr">
         <is>
-          <t>зубчик</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E792" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F792" s="2" t="inlineStr">
-        <is>
-          <t>измельчить</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="F792" s="2" t="n"/>
       <c r="G792" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H792" s="2" t="inlineStr">
@@ -33388,11 +33392,11 @@
       </c>
       <c r="B793" s="2" t="inlineStr">
         <is>
-          <t>лук</t>
+          <t>пассата</t>
         </is>
       </c>
       <c r="C793" s="2" t="n">
-        <v>40</v>
+        <v>85</v>
       </c>
       <c r="D793" s="2" t="inlineStr">
         <is>
@@ -33400,11 +33404,11 @@
         </is>
       </c>
       <c r="E793" s="2" t="n">
-        <v>40</v>
+        <v>85</v>
       </c>
       <c r="F793" s="2" t="inlineStr">
         <is>
-          <t>мелко нарезать</t>
+          <t>tomato sauce normalized to passata + spices policy</t>
         </is>
       </c>
       <c r="G793" s="2" t="inlineStr">
@@ -33414,7 +33418,7 @@
       </c>
       <c r="H793" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>prepared tomato sauce normalized to passata by user-approved tomato sauce policy</t>
         </is>
       </c>
     </row>
@@ -33426,21 +33430,25 @@
       </c>
       <c r="B794" s="2" t="inlineStr">
         <is>
-          <t>оливковое масло</t>
+          <t>чеснок</t>
         </is>
       </c>
       <c r="C794" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D794" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>зубчик</t>
         </is>
       </c>
       <c r="E794" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="F794" s="2" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="F794" s="2" t="inlineStr">
+        <is>
+          <t>измельчить</t>
+        </is>
+      </c>
       <c r="G794" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -33460,11 +33468,11 @@
       </c>
       <c r="B795" s="2" t="inlineStr">
         <is>
-          <t>сахар</t>
+          <t>лук</t>
         </is>
       </c>
       <c r="C795" s="2" t="n">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="D795" s="2" t="inlineStr">
         <is>
@@ -33472,11 +33480,11 @@
         </is>
       </c>
       <c r="E795" s="2" t="n">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="F795" s="2" t="inlineStr">
         <is>
-          <t>щепотка</t>
+          <t>мелко нарезать</t>
         </is>
       </c>
       <c r="G795" s="2" t="inlineStr">
@@ -33486,7 +33494,7 @@
       </c>
       <c r="H795" s="2" t="inlineStr">
         <is>
-          <t>normalized in validated cleanup slice</t>
+          <t>scaled from source</t>
         </is>
       </c>
     </row>
@@ -33498,41 +33506,45 @@
       </c>
       <c r="B796" s="2" t="inlineStr">
         <is>
-          <t>соль и перец</t>
-        </is>
-      </c>
-      <c r="C796" s="2" t="inlineStr">
-        <is>
-          <t>по вкусу</t>
-        </is>
+          <t>оливковое масло</t>
+        </is>
+      </c>
+      <c r="C796" s="2" t="n">
+        <v>8</v>
       </c>
       <c r="D796" s="2" t="inlineStr">
         <is>
-          <t>по вкусу</t>
-        </is>
-      </c>
-      <c r="E796" s="2" t="n"/>
+          <t>мл</t>
+        </is>
+      </c>
+      <c r="E796" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="F796" s="2" t="n"/>
       <c r="G796" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H796" s="2" t="n"/>
+      <c r="H796" s="2" t="inlineStr">
+        <is>
+          <t>scaled from source</t>
+        </is>
+      </c>
     </row>
     <row r="797">
       <c r="A797" s="2" t="inlineStr">
         <is>
-          <t>intake_101</t>
+          <t>intake_100</t>
         </is>
       </c>
       <c r="B797" s="2" t="inlineStr">
         <is>
-          <t>цельнозерновая паста</t>
+          <t>сахар</t>
         </is>
       </c>
       <c r="C797" s="2" t="n">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="D797" s="2" t="inlineStr">
         <is>
@@ -33540,9 +33552,13 @@
         </is>
       </c>
       <c r="E797" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F797" s="2" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="F797" s="2" t="inlineStr">
+        <is>
+          <t>щепотка</t>
+        </is>
+      </c>
       <c r="G797" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -33550,47 +33566,39 @@
       </c>
       <c r="H797" s="2" t="inlineStr">
         <is>
-          <t>scaled from source; normalized in validated cleanup slice</t>
+          <t>normalized in validated cleanup slice</t>
         </is>
       </c>
     </row>
     <row r="798">
       <c r="A798" s="2" t="inlineStr">
         <is>
-          <t>intake_101</t>
+          <t>intake_100</t>
         </is>
       </c>
       <c r="B798" s="2" t="inlineStr">
         <is>
-          <t>куриное филе</t>
-        </is>
-      </c>
-      <c r="C798" s="2" t="n">
-        <v>100</v>
+          <t>соль и перец</t>
+        </is>
+      </c>
+      <c r="C798" s="2" t="inlineStr">
+        <is>
+          <t>по вкусу</t>
+        </is>
       </c>
       <c r="D798" s="2" t="inlineStr">
         <is>
-          <t>г</t>
-        </is>
-      </c>
-      <c r="E798" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F798" s="2" t="inlineStr">
-        <is>
-          <t>кусочками, replaces processed poultry product by user decision</t>
-        </is>
-      </c>
+          <t>по вкусу</t>
+        </is>
+      </c>
+      <c r="E798" s="2" t="n"/>
+      <c r="F798" s="2" t="n"/>
       <c r="G798" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H798" s="2" t="inlineStr">
-        <is>
-          <t>processed poultry product replaced with chicken fillet by user decision</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H798" s="2" t="n"/>
     </row>
     <row r="799">
       <c r="A799" s="2" t="inlineStr">
@@ -33600,11 +33608,11 @@
       </c>
       <c r="B799" s="2" t="inlineStr">
         <is>
-          <t>пассата</t>
+          <t>цельнозерновая паста</t>
         </is>
       </c>
       <c r="C799" s="2" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="D799" s="2" t="inlineStr">
         <is>
@@ -33612,13 +33620,9 @@
         </is>
       </c>
       <c r="E799" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="F799" s="2" t="inlineStr">
-        <is>
-          <t>arrabbiata normalized to passata + chili/spices policy</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="F799" s="2" t="n"/>
       <c r="G799" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -33626,7 +33630,7 @@
       </c>
       <c r="H799" s="2" t="inlineStr">
         <is>
-          <t>prepared arrabbiata sauce normalized to passata by user-approved tomato sauce policy</t>
+          <t>scaled from source; normalized in validated cleanup slice</t>
         </is>
       </c>
     </row>
@@ -33638,29 +33642,33 @@
       </c>
       <c r="B800" s="2" t="inlineStr">
         <is>
-          <t>оливковое масло</t>
+          <t>куриное филе</t>
         </is>
       </c>
       <c r="C800" s="2" t="n">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="D800" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E800" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F800" s="2" t="n"/>
+        <v>100</v>
+      </c>
+      <c r="F800" s="2" t="inlineStr">
+        <is>
+          <t>кусочками, replaces processed poultry product by user decision</t>
+        </is>
+      </c>
       <c r="G800" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H800" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>processed poultry product replaced with chicken fillet by user decision</t>
         </is>
       </c>
     </row>
@@ -33672,7 +33680,7 @@
       </c>
       <c r="B801" s="2" t="inlineStr">
         <is>
-          <t>сладкий перец</t>
+          <t>пассата</t>
         </is>
       </c>
       <c r="C801" s="2" t="n">
@@ -33688,7 +33696,7 @@
       </c>
       <c r="F801" s="2" t="inlineStr">
         <is>
-          <t>вместо рамиро</t>
+          <t>arrabbiata normalized to passata + chili/spices policy</t>
         </is>
       </c>
       <c r="G801" s="2" t="inlineStr">
@@ -33698,7 +33706,7 @@
       </c>
       <c r="H801" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>prepared arrabbiata sauce normalized to passata by user-approved tomato sauce policy</t>
         </is>
       </c>
     </row>
@@ -33710,25 +33718,21 @@
       </c>
       <c r="B802" s="2" t="inlineStr">
         <is>
-          <t>лук</t>
+          <t>оливковое масло</t>
         </is>
       </c>
       <c r="C802" s="2" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="D802" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>мл</t>
         </is>
       </c>
       <c r="E802" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="F802" s="2" t="inlineStr">
-        <is>
-          <t>мелко нарезать</t>
-        </is>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F802" s="2" t="n"/>
       <c r="G802" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -33748,23 +33752,23 @@
       </c>
       <c r="B803" s="2" t="inlineStr">
         <is>
-          <t>чеснок</t>
+          <t>сладкий перец</t>
         </is>
       </c>
       <c r="C803" s="2" t="n">
-        <v>1</v>
+        <v>75</v>
       </c>
       <c r="D803" s="2" t="inlineStr">
         <is>
-          <t>зубчик</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E803" s="2" t="n">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="F803" s="2" t="inlineStr">
         <is>
-          <t>измельчить</t>
+          <t>вместо рамиро</t>
         </is>
       </c>
       <c r="G803" s="2" t="inlineStr">
@@ -33786,11 +33790,11 @@
       </c>
       <c r="B804" s="2" t="inlineStr">
         <is>
-          <t>пармезан</t>
+          <t>лук</t>
         </is>
       </c>
       <c r="C804" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D804" s="2" t="inlineStr">
         <is>
@@ -33798,16 +33802,16 @@
         </is>
       </c>
       <c r="E804" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F804" s="2" t="inlineStr">
         <is>
-          <t>для подачи</t>
+          <t>мелко нарезать</t>
         </is>
       </c>
       <c r="G804" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H804" s="2" t="inlineStr">
@@ -33824,23 +33828,23 @@
       </c>
       <c r="B805" s="2" t="inlineStr">
         <is>
-          <t>базилик</t>
+          <t>чеснок</t>
         </is>
       </c>
       <c r="C805" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D805" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>зубчик</t>
         </is>
       </c>
       <c r="E805" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F805" s="2" t="inlineStr">
         <is>
-          <t>для подачи</t>
+          <t>измельчить</t>
         </is>
       </c>
       <c r="G805" s="2" t="inlineStr">
@@ -33862,45 +33866,49 @@
       </c>
       <c r="B806" s="2" t="inlineStr">
         <is>
-          <t>соль, перец, сахар, чили</t>
-        </is>
-      </c>
-      <c r="C806" s="2" t="inlineStr">
-        <is>
-          <t>по вкусу</t>
-        </is>
+          <t>пармезан</t>
+        </is>
+      </c>
+      <c r="C806" s="2" t="n">
+        <v>20</v>
       </c>
       <c r="D806" s="2" t="inlineStr">
         <is>
-          <t>по вкусу</t>
-        </is>
-      </c>
-      <c r="E806" s="2" t="n"/>
-      <c r="F806" s="2" t="n"/>
+          <t>г</t>
+        </is>
+      </c>
+      <c r="E806" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F806" s="2" t="inlineStr">
+        <is>
+          <t>для подачи</t>
+        </is>
+      </c>
       <c r="G806" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H806" s="2" t="inlineStr">
         <is>
-          <t>chili/spices retained for arrabbiata flavor after passata normalization</t>
+          <t>scaled from source</t>
         </is>
       </c>
     </row>
     <row r="807">
       <c r="A807" s="2" t="inlineStr">
         <is>
-          <t>intake_102</t>
+          <t>intake_101</t>
         </is>
       </c>
       <c r="B807" s="2" t="inlineStr">
         <is>
-          <t>цельнозерновая паста</t>
+          <t>базилик</t>
         </is>
       </c>
       <c r="C807" s="2" t="n">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="D807" s="2" t="inlineStr">
         <is>
@@ -33908,9 +33916,13 @@
         </is>
       </c>
       <c r="E807" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F807" s="2" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="F807" s="2" t="inlineStr">
+        <is>
+          <t>для подачи</t>
+        </is>
+      </c>
       <c r="G807" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -33918,45 +33930,41 @@
       </c>
       <c r="H807" s="2" t="inlineStr">
         <is>
-          <t>scaled from source; normalized in validated cleanup slice</t>
+          <t>scaled from source</t>
         </is>
       </c>
     </row>
     <row r="808">
       <c r="A808" s="2" t="inlineStr">
         <is>
-          <t>intake_102</t>
+          <t>intake_101</t>
         </is>
       </c>
       <c r="B808" s="2" t="inlineStr">
         <is>
-          <t>лосось</t>
-        </is>
-      </c>
-      <c r="C808" s="2" t="n">
-        <v>100</v>
+          <t>соль, перец, сахар, чили</t>
+        </is>
+      </c>
+      <c r="C808" s="2" t="inlineStr">
+        <is>
+          <t>по вкусу</t>
+        </is>
       </c>
       <c r="D808" s="2" t="inlineStr">
         <is>
-          <t>г</t>
-        </is>
-      </c>
-      <c r="E808" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F808" s="2" t="inlineStr">
-        <is>
-          <t>кусочками</t>
-        </is>
-      </c>
+          <t>по вкусу</t>
+        </is>
+      </c>
+      <c r="E808" s="2" t="n"/>
+      <c r="F808" s="2" t="n"/>
       <c r="G808" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H808" s="2" t="inlineStr">
         <is>
-          <t>scaled from source; normalized in validated cleanup slice</t>
+          <t>chili/spices retained for arrabbiata flavor after passata normalization</t>
         </is>
       </c>
     </row>
@@ -33968,7 +33976,7 @@
       </c>
       <c r="B809" s="2" t="inlineStr">
         <is>
-          <t>сливки 10%</t>
+          <t>цельнозерновая паста</t>
         </is>
       </c>
       <c r="C809" s="2" t="n">
@@ -33976,7 +33984,7 @@
       </c>
       <c r="D809" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E809" s="2" t="n">
@@ -33990,7 +33998,7 @@
       </c>
       <c r="H809" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>scaled from source; normalized in validated cleanup slice</t>
         </is>
       </c>
     </row>
@@ -34002,11 +34010,11 @@
       </c>
       <c r="B810" s="2" t="inlineStr">
         <is>
-          <t>шпинат</t>
+          <t>лосось</t>
         </is>
       </c>
       <c r="C810" s="2" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D810" s="2" t="inlineStr">
         <is>
@@ -34014,17 +34022,21 @@
         </is>
       </c>
       <c r="E810" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="F810" s="2" t="n"/>
+        <v>100</v>
+      </c>
+      <c r="F810" s="2" t="inlineStr">
+        <is>
+          <t>кусочками</t>
+        </is>
+      </c>
       <c r="G810" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H810" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>scaled from source; normalized in validated cleanup slice</t>
         </is>
       </c>
     </row>
@@ -34036,19 +34048,19 @@
       </c>
       <c r="B811" s="2" t="inlineStr">
         <is>
-          <t>творожный сыр</t>
+          <t>сливки 10%</t>
         </is>
       </c>
       <c r="C811" s="2" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="D811" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>мл</t>
         </is>
       </c>
       <c r="E811" s="2" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="F811" s="2" t="n"/>
       <c r="G811" s="2" t="inlineStr">
@@ -34070,19 +34082,19 @@
       </c>
       <c r="B812" s="2" t="inlineStr">
         <is>
-          <t>оливковое масло</t>
+          <t>шпинат</t>
         </is>
       </c>
       <c r="C812" s="2" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="D812" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E812" s="2" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="F812" s="2" t="n"/>
       <c r="G812" s="2" t="inlineStr">
@@ -34104,25 +34116,21 @@
       </c>
       <c r="B813" s="2" t="inlineStr">
         <is>
-          <t>чеснок</t>
+          <t>творожный сыр</t>
         </is>
       </c>
       <c r="C813" s="2" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="D813" s="2" t="inlineStr">
         <is>
-          <t>зубчик</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E813" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F813" s="2" t="inlineStr">
-        <is>
-          <t>измельчить</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="F813" s="2" t="n"/>
       <c r="G813" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -34142,28 +34150,24 @@
       </c>
       <c r="B814" s="2" t="inlineStr">
         <is>
-          <t>пармезан</t>
+          <t>оливковое масло</t>
         </is>
       </c>
       <c r="C814" s="2" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D814" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>мл</t>
         </is>
       </c>
       <c r="E814" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="F814" s="2" t="inlineStr">
-        <is>
-          <t>для подачи</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="F814" s="2" t="n"/>
       <c r="G814" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H814" s="2" t="inlineStr">
@@ -34180,23 +34184,23 @@
       </c>
       <c r="B815" s="2" t="inlineStr">
         <is>
-          <t>базилик</t>
+          <t>чеснок</t>
         </is>
       </c>
       <c r="C815" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D815" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>зубчик</t>
         </is>
       </c>
       <c r="E815" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F815" s="2" t="inlineStr">
         <is>
-          <t>для подачи</t>
+          <t>измельчить</t>
         </is>
       </c>
       <c r="G815" s="2" t="inlineStr">
@@ -34218,41 +34222,49 @@
       </c>
       <c r="B816" s="2" t="inlineStr">
         <is>
-          <t>соль, перец, сахар</t>
-        </is>
-      </c>
-      <c r="C816" s="2" t="inlineStr">
-        <is>
-          <t>по вкусу</t>
-        </is>
+          <t>пармезан</t>
+        </is>
+      </c>
+      <c r="C816" s="2" t="n">
+        <v>20</v>
       </c>
       <c r="D816" s="2" t="inlineStr">
         <is>
-          <t>по вкусу</t>
-        </is>
-      </c>
-      <c r="E816" s="2" t="n"/>
-      <c r="F816" s="2" t="n"/>
+          <t>г</t>
+        </is>
+      </c>
+      <c r="E816" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F816" s="2" t="inlineStr">
+        <is>
+          <t>для подачи</t>
+        </is>
+      </c>
       <c r="G816" s="2" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H816" s="2" t="n"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H816" s="2" t="inlineStr">
+        <is>
+          <t>scaled from source</t>
+        </is>
+      </c>
     </row>
     <row r="817">
       <c r="A817" s="2" t="inlineStr">
         <is>
-          <t>intake_103</t>
+          <t>intake_102</t>
         </is>
       </c>
       <c r="B817" s="2" t="inlineStr">
         <is>
-          <t>макароны</t>
+          <t>базилик</t>
         </is>
       </c>
       <c r="C817" s="2" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="D817" s="2" t="inlineStr">
         <is>
@@ -34260,9 +34272,13 @@
         </is>
       </c>
       <c r="E817" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="F817" s="2" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="F817" s="2" t="inlineStr">
+        <is>
+          <t>для подачи</t>
+        </is>
+      </c>
       <c r="G817" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -34277,36 +34293,32 @@
     <row r="818">
       <c r="A818" s="2" t="inlineStr">
         <is>
-          <t>intake_103</t>
+          <t>intake_102</t>
         </is>
       </c>
       <c r="B818" s="2" t="inlineStr">
         <is>
-          <t>молоко</t>
-        </is>
-      </c>
-      <c r="C818" s="2" t="n">
-        <v>80</v>
+          <t>соль, перец, сахар</t>
+        </is>
+      </c>
+      <c r="C818" s="2" t="inlineStr">
+        <is>
+          <t>по вкусу</t>
+        </is>
       </c>
       <c r="D818" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
-        </is>
-      </c>
-      <c r="E818" s="2" t="n">
-        <v>80</v>
-      </c>
+          <t>по вкусу</t>
+        </is>
+      </c>
+      <c r="E818" s="2" t="n"/>
       <c r="F818" s="2" t="n"/>
       <c r="G818" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H818" s="2" t="inlineStr">
-        <is>
-          <t>scaled from source</t>
-        </is>
-      </c>
+      <c r="H818" s="2" t="n"/>
     </row>
     <row r="819">
       <c r="A819" s="2" t="inlineStr">
@@ -34316,11 +34328,11 @@
       </c>
       <c r="B819" s="2" t="inlineStr">
         <is>
-          <t>сыр чеддер</t>
+          <t>макароны</t>
         </is>
       </c>
       <c r="C819" s="2" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="D819" s="2" t="inlineStr">
         <is>
@@ -34328,16 +34340,12 @@
         </is>
       </c>
       <c r="E819" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="F819" s="2" t="inlineStr">
-        <is>
-          <t>натереть</t>
-        </is>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="F819" s="2" t="n"/>
       <c r="G819" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H819" s="2" t="inlineStr">
@@ -34354,28 +34362,24 @@
       </c>
       <c r="B820" s="2" t="inlineStr">
         <is>
-          <t>моцарелла</t>
+          <t>молоко</t>
         </is>
       </c>
       <c r="C820" s="2" t="n">
-        <v>35</v>
+        <v>80</v>
       </c>
       <c r="D820" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>мл</t>
         </is>
       </c>
       <c r="E820" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="F820" s="2" t="inlineStr">
-        <is>
-          <t>натереть</t>
-        </is>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="F820" s="2" t="n"/>
       <c r="G820" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H820" s="2" t="inlineStr">
@@ -34392,11 +34396,11 @@
       </c>
       <c r="B821" s="2" t="inlineStr">
         <is>
-          <t>мука</t>
+          <t>сыр чеддер</t>
         </is>
       </c>
       <c r="C821" s="2" t="n">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="D821" s="2" t="inlineStr">
         <is>
@@ -34404,12 +34408,16 @@
         </is>
       </c>
       <c r="E821" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F821" s="2" t="n"/>
+        <v>70</v>
+      </c>
+      <c r="F821" s="2" t="inlineStr">
+        <is>
+          <t>натереть</t>
+        </is>
+      </c>
       <c r="G821" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H821" s="2" t="inlineStr">
@@ -34426,11 +34434,11 @@
       </c>
       <c r="B822" s="2" t="inlineStr">
         <is>
-          <t>сливочное масло</t>
+          <t>моцарелла</t>
         </is>
       </c>
       <c r="C822" s="2" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="D822" s="2" t="inlineStr">
         <is>
@@ -34438,12 +34446,16 @@
         </is>
       </c>
       <c r="E822" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F822" s="2" t="n"/>
+        <v>35</v>
+      </c>
+      <c r="F822" s="2" t="inlineStr">
+        <is>
+          <t>натереть</t>
+        </is>
+      </c>
       <c r="G822" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H822" s="2" t="inlineStr">
@@ -34460,41 +34472,45 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>соль и перец</t>
-        </is>
-      </c>
-      <c r="C823" s="2" t="inlineStr">
-        <is>
-          <t>по вкусу</t>
-        </is>
+          <t>мука</t>
+        </is>
+      </c>
+      <c r="C823" s="2" t="n">
+        <v>15</v>
       </c>
       <c r="D823" s="2" t="inlineStr">
         <is>
-          <t>по вкусу</t>
-        </is>
-      </c>
-      <c r="E823" s="2" t="n"/>
+          <t>г</t>
+        </is>
+      </c>
+      <c r="E823" s="2" t="n">
+        <v>15</v>
+      </c>
       <c r="F823" s="2" t="n"/>
       <c r="G823" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H823" s="2" t="n"/>
+      <c r="H823" s="2" t="inlineStr">
+        <is>
+          <t>scaled from source</t>
+        </is>
+      </c>
     </row>
     <row r="824">
       <c r="A824" s="2" t="inlineStr">
         <is>
-          <t>intake_104</t>
+          <t>intake_103</t>
         </is>
       </c>
       <c r="B824" s="2" t="inlineStr">
         <is>
-          <t>говяжий фарш</t>
+          <t>сливочное масло</t>
         </is>
       </c>
       <c r="C824" s="2" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="D824" s="2" t="inlineStr">
         <is>
@@ -34502,12 +34518,12 @@
         </is>
       </c>
       <c r="E824" s="2" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="F824" s="2" t="n"/>
       <c r="G824" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H824" s="2" t="inlineStr">
@@ -34519,36 +34535,32 @@
     <row r="825">
       <c r="A825" s="2" t="inlineStr">
         <is>
-          <t>intake_104</t>
+          <t>intake_103</t>
         </is>
       </c>
       <c r="B825" s="2" t="inlineStr">
         <is>
-          <t>цельнозерновая паста</t>
-        </is>
-      </c>
-      <c r="C825" s="2" t="n">
-        <v>50</v>
+          <t>соль и перец</t>
+        </is>
+      </c>
+      <c r="C825" s="2" t="inlineStr">
+        <is>
+          <t>по вкусу</t>
+        </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
         <is>
-          <t>г</t>
-        </is>
-      </c>
-      <c r="E825" s="2" t="n">
-        <v>50</v>
-      </c>
+          <t>по вкусу</t>
+        </is>
+      </c>
+      <c r="E825" s="2" t="n"/>
       <c r="F825" s="2" t="n"/>
       <c r="G825" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H825" s="2" t="inlineStr">
-        <is>
-          <t>scaled from source; normalized in validated cleanup slice</t>
-        </is>
-      </c>
+      <c r="H825" s="2" t="n"/>
     </row>
     <row r="826">
       <c r="A826" s="2" t="inlineStr">
@@ -34558,11 +34570,11 @@
       </c>
       <c r="B826" s="2" t="inlineStr">
         <is>
-          <t>резаные томаты</t>
+          <t>говяжий фарш</t>
         </is>
       </c>
       <c r="C826" s="2" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="D826" s="2" t="inlineStr">
         <is>
@@ -34570,21 +34582,17 @@
         </is>
       </c>
       <c r="E826" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="F826" s="2" t="inlineStr">
-        <is>
-          <t>в собственном соку</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="F826" s="2" t="n"/>
       <c r="G826" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H826" s="2" t="inlineStr">
         <is>
-          <t>chopped/canned tomatoes mapping readiness confirmed by user-approved tomato variant policy</t>
+          <t>scaled from source</t>
         </is>
       </c>
     </row>
@@ -34596,11 +34604,11 @@
       </c>
       <c r="B827" s="2" t="inlineStr">
         <is>
-          <t>сыр гауда</t>
+          <t>цельнозерновая паста</t>
         </is>
       </c>
       <c r="C827" s="2" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D827" s="2" t="inlineStr">
         <is>
@@ -34608,16 +34616,12 @@
         </is>
       </c>
       <c r="E827" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="F827" s="2" t="inlineStr">
-        <is>
-          <t>натереть</t>
-        </is>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="F827" s="2" t="n"/>
       <c r="G827" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H827" s="2" t="inlineStr">
@@ -34634,11 +34638,11 @@
       </c>
       <c r="B828" s="2" t="inlineStr">
         <is>
-          <t>маринованный огурец</t>
+          <t>резаные томаты</t>
         </is>
       </c>
       <c r="C828" s="2" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="D828" s="2" t="inlineStr">
         <is>
@@ -34646,11 +34650,11 @@
         </is>
       </c>
       <c r="E828" s="2" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="F828" s="2" t="inlineStr">
         <is>
-          <t>кубиками</t>
+          <t>в собственном соку</t>
         </is>
       </c>
       <c r="G828" s="2" t="inlineStr">
@@ -34660,7 +34664,7 @@
       </c>
       <c r="H828" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>chopped/canned tomatoes mapping readiness confirmed by user-approved tomato variant policy</t>
         </is>
       </c>
     </row>
@@ -34672,11 +34676,11 @@
       </c>
       <c r="B829" s="2" t="inlineStr">
         <is>
-          <t>морковь</t>
+          <t>сыр гауда</t>
         </is>
       </c>
       <c r="C829" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D829" s="2" t="inlineStr">
         <is>
@@ -34684,7 +34688,7 @@
         </is>
       </c>
       <c r="E829" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F829" s="2" t="inlineStr">
         <is>
@@ -34693,12 +34697,12 @@
       </c>
       <c r="G829" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H829" s="2" t="inlineStr">
         <is>
-          <t>scaled from source</t>
+          <t>scaled from source; normalized in validated cleanup slice</t>
         </is>
       </c>
     </row>
@@ -34710,11 +34714,11 @@
       </c>
       <c r="B830" s="2" t="inlineStr">
         <is>
-          <t>лук</t>
+          <t>маринованный огурец</t>
         </is>
       </c>
       <c r="C830" s="2" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="D830" s="2" t="inlineStr">
         <is>
@@ -34722,11 +34726,11 @@
         </is>
       </c>
       <c r="E830" s="2" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="F830" s="2" t="inlineStr">
         <is>
-          <t>мелко нарезать</t>
+          <t>кубиками</t>
         </is>
       </c>
       <c r="G830" s="2" t="inlineStr">
@@ -34748,21 +34752,25 @@
       </c>
       <c r="B831" s="2" t="inlineStr">
         <is>
-          <t>растительное масло</t>
+          <t>морковь</t>
         </is>
       </c>
       <c r="C831" s="2" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="D831" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E831" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="F831" s="2" t="n"/>
+        <v>30</v>
+      </c>
+      <c r="F831" s="2" t="inlineStr">
+        <is>
+          <t>натереть</t>
+        </is>
+      </c>
       <c r="G831" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -34782,25 +34790,23 @@
       </c>
       <c r="B832" s="2" t="inlineStr">
         <is>
-          <t>специи</t>
-        </is>
-      </c>
-      <c r="C832" s="2" t="inlineStr">
-        <is>
-          <t>1/4</t>
-        </is>
+          <t>лук</t>
+        </is>
+      </c>
+      <c r="C832" s="2" t="n">
+        <v>25</v>
       </c>
       <c r="D832" s="2" t="inlineStr">
         <is>
-          <t>ч. л.</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E832" s="2" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="F832" s="2" t="inlineStr">
         <is>
-          <t>хмели-сунели</t>
+          <t>мелко нарезать</t>
         </is>
       </c>
       <c r="G832" s="2" t="inlineStr">
@@ -34810,7 +34816,7 @@
       </c>
       <c r="H832" s="2" t="inlineStr">
         <is>
-          <t>khmeli-suneli mapped to mixed_spices by user decision</t>
+          <t>scaled from source</t>
         </is>
       </c>
     </row>
@@ -34822,53 +34828,59 @@
       </c>
       <c r="B833" s="2" t="inlineStr">
         <is>
-          <t>соль, перец, зелень</t>
-        </is>
-      </c>
-      <c r="C833" s="2" t="inlineStr">
-        <is>
-          <t>по вкусу</t>
-        </is>
+          <t>растительное масло</t>
+        </is>
+      </c>
+      <c r="C833" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="D833" s="2" t="inlineStr">
         <is>
-          <t>по вкусу</t>
-        </is>
-      </c>
-      <c r="E833" s="2" t="n"/>
+          <t>мл</t>
+        </is>
+      </c>
+      <c r="E833" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="F833" s="2" t="n"/>
       <c r="G833" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H833" s="2" t="n"/>
+      <c r="H833" s="2" t="inlineStr">
+        <is>
+          <t>scaled from source</t>
+        </is>
+      </c>
     </row>
     <row r="834">
       <c r="A834" s="2" t="inlineStr">
         <is>
-          <t>intake_105</t>
+          <t>intake_104</t>
         </is>
       </c>
       <c r="B834" s="2" t="inlineStr">
         <is>
-          <t>зеленый горошек</t>
-        </is>
-      </c>
-      <c r="C834" s="2" t="n">
-        <v>100</v>
+          <t>специи</t>
+        </is>
+      </c>
+      <c r="C834" s="2" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
       </c>
       <c r="D834" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>ч. л.</t>
         </is>
       </c>
       <c r="E834" s="2" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F834" s="2" t="inlineStr">
         <is>
-          <t>вместо эдамамэ</t>
+          <t>хмели-сунели</t>
         </is>
       </c>
       <c r="G834" s="2" t="inlineStr">
@@ -34878,47 +34890,39 @@
       </c>
       <c r="H834" s="2" t="inlineStr">
         <is>
-          <t>accessible replacement</t>
+          <t>khmeli-suneli mapped to mixed_spices by user decision</t>
         </is>
       </c>
     </row>
     <row r="835">
       <c r="A835" s="2" t="inlineStr">
         <is>
-          <t>intake_105</t>
+          <t>intake_104</t>
         </is>
       </c>
       <c r="B835" s="2" t="inlineStr">
         <is>
-          <t>картофель</t>
-        </is>
-      </c>
-      <c r="C835" s="2" t="n">
-        <v>125</v>
+          <t>соль, перец, зелень</t>
+        </is>
+      </c>
+      <c r="C835" s="2" t="inlineStr">
+        <is>
+          <t>по вкусу</t>
+        </is>
       </c>
       <c r="D835" s="2" t="inlineStr">
         <is>
-          <t>г</t>
-        </is>
-      </c>
-      <c r="E835" s="2" t="n">
-        <v>125</v>
-      </c>
-      <c r="F835" s="2" t="inlineStr">
-        <is>
-          <t>кубиками</t>
-        </is>
-      </c>
+          <t>по вкусу</t>
+        </is>
+      </c>
+      <c r="E835" s="2" t="n"/>
+      <c r="F835" s="2" t="n"/>
       <c r="G835" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H835" s="2" t="inlineStr">
-        <is>
-          <t>from source</t>
-        </is>
-      </c>
+      <c r="H835" s="2" t="n"/>
     </row>
     <row r="836">
       <c r="A836" s="2" t="inlineStr">
@@ -34928,11 +34932,11 @@
       </c>
       <c r="B836" s="2" t="inlineStr">
         <is>
-          <t>креветки очищенные</t>
+          <t>зеленый горошек</t>
         </is>
       </c>
       <c r="C836" s="2" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D836" s="2" t="inlineStr">
         <is>
@@ -34940,16 +34944,16 @@
         </is>
       </c>
       <c r="E836" s="2" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="F836" s="2" t="inlineStr">
         <is>
-          <t>вместо морских гребешков</t>
+          <t>вместо эдамамэ</t>
         </is>
       </c>
       <c r="G836" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H836" s="2" t="inlineStr">
@@ -34966,11 +34970,11 @@
       </c>
       <c r="B837" s="2" t="inlineStr">
         <is>
-          <t>соус терияки</t>
+          <t>картофель</t>
         </is>
       </c>
       <c r="C837" s="2" t="n">
-        <v>15</v>
+        <v>125</v>
       </c>
       <c r="D837" s="2" t="inlineStr">
         <is>
@@ -34978,9 +34982,13 @@
         </is>
       </c>
       <c r="E837" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F837" s="2" t="n"/>
+        <v>125</v>
+      </c>
+      <c r="F837" s="2" t="inlineStr">
+        <is>
+          <t>кубиками</t>
+        </is>
+      </c>
       <c r="G837" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -34988,7 +34996,7 @@
       </c>
       <c r="H837" s="2" t="inlineStr">
         <is>
-          <t>from source; teriyaki policy approved with modest explicit grams; low-confidence sodium/sugar note acceptable</t>
+          <t>from source</t>
         </is>
       </c>
     </row>
@@ -35000,28 +35008,28 @@
       </c>
       <c r="B838" s="2" t="inlineStr">
         <is>
-          <t>сливки 20%</t>
+          <t>креветки очищенные</t>
         </is>
       </c>
       <c r="C838" s="2" t="n">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="D838" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E838" s="2" t="n">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="F838" s="2" t="inlineStr">
         <is>
-          <t>вместо 38%</t>
+          <t>вместо морских гребешков</t>
         </is>
       </c>
       <c r="G838" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H838" s="2" t="inlineStr">
@@ -35038,11 +35046,11 @@
       </c>
       <c r="B839" s="2" t="inlineStr">
         <is>
-          <t>репчатый лук</t>
+          <t>соус терияки</t>
         </is>
       </c>
       <c r="C839" s="2" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D839" s="2" t="inlineStr">
         <is>
@@ -35050,13 +35058,9 @@
         </is>
       </c>
       <c r="E839" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="F839" s="2" t="inlineStr">
-        <is>
-          <t>мелко нарезать</t>
-        </is>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F839" s="2" t="n"/>
       <c r="G839" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -35064,7 +35068,7 @@
       </c>
       <c r="H839" s="2" t="inlineStr">
         <is>
-          <t>from source</t>
+          <t>from source; teriyaki policy approved with modest explicit grams; low-confidence sodium/sugar note acceptable</t>
         </is>
       </c>
     </row>
@@ -35076,23 +35080,23 @@
       </c>
       <c r="B840" s="2" t="inlineStr">
         <is>
-          <t>чеснок</t>
+          <t>сливки 20%</t>
         </is>
       </c>
       <c r="C840" s="2" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D840" s="2" t="inlineStr">
         <is>
-          <t>г</t>
+          <t>мл</t>
         </is>
       </c>
       <c r="E840" s="2" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F840" s="2" t="inlineStr">
         <is>
-          <t>измельчить</t>
+          <t>вместо 38%</t>
         </is>
       </c>
       <c r="G840" s="2" t="inlineStr">
@@ -35102,7 +35106,7 @@
       </c>
       <c r="H840" s="2" t="inlineStr">
         <is>
-          <t>from source</t>
+          <t>accessible replacement</t>
         </is>
       </c>
     </row>
@@ -35114,11 +35118,11 @@
       </c>
       <c r="B841" s="2" t="inlineStr">
         <is>
-          <t>сельдерей стеблевой</t>
+          <t>репчатый лук</t>
         </is>
       </c>
       <c r="C841" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D841" s="2" t="inlineStr">
         <is>
@@ -35126,11 +35130,11 @@
         </is>
       </c>
       <c r="E841" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F841" s="2" t="inlineStr">
         <is>
-          <t>тонко нарезать</t>
+          <t>мелко нарезать</t>
         </is>
       </c>
       <c r="G841" s="2" t="inlineStr">
@@ -35152,11 +35156,11 @@
       </c>
       <c r="B842" s="2" t="inlineStr">
         <is>
-          <t>кедровые орехи</t>
+          <t>чеснок</t>
         </is>
       </c>
       <c r="C842" s="2" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D842" s="2" t="inlineStr">
         <is>
@@ -35164,11 +35168,11 @@
         </is>
       </c>
       <c r="E842" s="2" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F842" s="2" t="inlineStr">
         <is>
-          <t>слегка обжарить</t>
+          <t>измельчить</t>
         </is>
       </c>
       <c r="G842" s="2" t="inlineStr">
@@ -35190,11 +35194,11 @@
       </c>
       <c r="B843" s="2" t="inlineStr">
         <is>
-          <t>сливочное масло</t>
+          <t>сельдерей стеблевой</t>
         </is>
       </c>
       <c r="C843" s="2" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D843" s="2" t="inlineStr">
         <is>
@@ -35202,9 +35206,13 @@
         </is>
       </c>
       <c r="E843" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F843" s="2" t="n"/>
+        <v>30</v>
+      </c>
+      <c r="F843" s="2" t="inlineStr">
+        <is>
+          <t>тонко нарезать</t>
+        </is>
+      </c>
       <c r="G843" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -35224,21 +35232,25 @@
       </c>
       <c r="B844" s="2" t="inlineStr">
         <is>
-          <t>растительное масло</t>
+          <t>кедровые орехи</t>
         </is>
       </c>
       <c r="C844" s="2" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D844" s="2" t="inlineStr">
         <is>
-          <t>мл</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E844" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F844" s="2" t="n"/>
+        <v>20</v>
+      </c>
+      <c r="F844" s="2" t="inlineStr">
+        <is>
+          <t>слегка обжарить</t>
+        </is>
+      </c>
       <c r="G844" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -35258,41 +35270,45 @@
       </c>
       <c r="B845" s="2" t="inlineStr">
         <is>
-          <t>соль и перец</t>
-        </is>
-      </c>
-      <c r="C845" s="2" t="inlineStr">
-        <is>
-          <t>по вкусу</t>
-        </is>
+          <t>сливочное масло</t>
+        </is>
+      </c>
+      <c r="C845" s="2" t="n">
+        <v>10</v>
       </c>
       <c r="D845" s="2" t="inlineStr">
         <is>
-          <t>по вкусу</t>
-        </is>
-      </c>
-      <c r="E845" s="2" t="n"/>
+          <t>г</t>
+        </is>
+      </c>
+      <c r="E845" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="F845" s="2" t="n"/>
       <c r="G845" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="H845" s="2" t="n"/>
+      <c r="H845" s="2" t="inlineStr">
+        <is>
+          <t>from source</t>
+        </is>
+      </c>
     </row>
     <row r="846">
       <c r="A846" s="2" t="inlineStr">
         <is>
-          <t>intake_070</t>
+          <t>intake_105</t>
         </is>
       </c>
       <c r="B846" s="2" t="inlineStr">
         <is>
-          <t>вода</t>
+          <t>растительное масло</t>
         </is>
       </c>
       <c r="C846" s="2" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D846" s="2" t="inlineStr">
         <is>
@@ -35300,13 +35316,9 @@
         </is>
       </c>
       <c r="E846" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="F846" s="2" t="inlineStr">
-        <is>
-          <t>для кляра</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="F846" s="2" t="n"/>
       <c r="G846" s="2" t="inlineStr">
         <is>
           <t>no</t>
@@ -35314,19 +35326,87 @@
       </c>
       <c r="H846" s="2" t="inlineStr">
         <is>
-          <t>normalized in validated cleanup slice</t>
+          <t>from source</t>
         </is>
       </c>
     </row>
     <row r="847">
-      <c r="A847" s="2" t="n"/>
-      <c r="B847" s="2" t="n"/>
-      <c r="C847" s="2" t="n"/>
-      <c r="D847" s="2" t="n"/>
+      <c r="A847" s="2" t="inlineStr">
+        <is>
+          <t>intake_105</t>
+        </is>
+      </c>
+      <c r="B847" s="2" t="inlineStr">
+        <is>
+          <t>соль и перец</t>
+        </is>
+      </c>
+      <c r="C847" s="2" t="inlineStr">
+        <is>
+          <t>по вкусу</t>
+        </is>
+      </c>
+      <c r="D847" s="2" t="inlineStr">
+        <is>
+          <t>по вкусу</t>
+        </is>
+      </c>
       <c r="E847" s="2" t="n"/>
       <c r="F847" s="2" t="n"/>
-      <c r="G847" s="2" t="n"/>
+      <c r="G847" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="H847" s="2" t="n"/>
+    </row>
+    <row r="848">
+      <c r="A848" s="2" t="inlineStr">
+        <is>
+          <t>intake_070</t>
+        </is>
+      </c>
+      <c r="B848" s="2" t="inlineStr">
+        <is>
+          <t>вода</t>
+        </is>
+      </c>
+      <c r="C848" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D848" s="2" t="inlineStr">
+        <is>
+          <t>мл</t>
+        </is>
+      </c>
+      <c r="E848" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F848" s="2" t="inlineStr">
+        <is>
+          <t>для кляра</t>
+        </is>
+      </c>
+      <c r="G848" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H848" s="2" t="inlineStr">
+        <is>
+          <t>normalized in validated cleanup slice</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="2" t="n"/>
+      <c r="B849" s="2" t="n"/>
+      <c r="C849" s="2" t="n"/>
+      <c r="D849" s="2" t="n"/>
+      <c r="E849" s="2" t="n"/>
+      <c r="F849" s="2" t="n"/>
+      <c r="G849" s="2" t="n"/>
+      <c r="H849" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -41333,7 +41413,7 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Замороженный фалафель поджарьте на сковороде, смазанной маслом, по 1,5—2 минуты с каждой стороны.</t>
+          <t>Замороженный фалафель поджарьте на сковороде, смазанной маслом, по 1,5-2 минуты с каждой стороны.</t>
         </is>
       </c>
     </row>
@@ -41348,7 +41428,7 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Помидоры нарежьте тонкими слайсами, огурцы — соломкой, лук мелко порубите.</t>
+          <t>Помидоры нарежьте тонкими слайсами, огурцы - соломкой, зеленый лук мелко порубите.</t>
         </is>
       </c>
     </row>
@@ -41363,7 +41443,7 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>На лист лаваша выложите половину овощей, 4 шарика фалафеля, половину соуса и заверните в шаурму.</t>
+          <t>Смешайте греческий йогурт, соевый соус и лимонный сок до однородного легкого соуса.</t>
         </is>
       </c>
     </row>
@@ -41378,7 +41458,7 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Подпеките шаурму с 2 сторон на сухой сковороде, разрежьте пополам и подавайте.</t>
+          <t>На лист лаваша выложите томаты, огурец, морковь по-корейски, фалафель и соус, заверните, подпеките с двух сторон на сухой сковороде, разрежьте пополам и подавайте.</t>
         </is>
       </c>
     </row>
@@ -46139,12 +46219,12 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Решение пользователя применено.</t>
+          <t>Финальное решение по risky-cleanup применено.</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Замороженный фалафель оставлен как полуфабрикат для staging; фалафель отмечен как растительный белковый anchor.</t>
+          <t>Фалафель и морковь по-корейски оставлены как accepted prepared products; готовый майонезно-соевый соус заменен на греческий йогурт 30 г, соевый соус 5 г и лимонный сок 5 г.</t>
         </is>
       </c>
     </row>

</xml_diff>